<commit_message>
Add bicycle infrastructure layers: bike lanes, Divvy stations, bike racks
- Bike Routes (37 features) from City of Chicago SODA API (hvv9-38ut)
- Divvy Stations (22 in boundary) from SODA API (bbyy-e7gq)
- Bike Racks (16 in boundary) from OpenStreetMap Overpass API
- Updated Folium map, Leaflet site, data.js, and Excel export
- New filter panel checkboxes, legend items, and layer rendering

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bronzeville_assets.xlsx
+++ b/bronzeville_assets.xlsx
@@ -21,6 +21,9 @@
     <sheet name="CTA Bus Routes" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Metra Stations" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Metra Lines" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Bike Routes" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Divvy Stations" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bike Racks" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,7 +46,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -95,6 +98,21 @@
         <fgColor rgb="001A5276"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000897B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001565C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004DD0E1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -113,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -140,6 +158,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -16345,6 +16372,3987 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>street</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>st_name</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>oneway_dir</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>f_street</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>t_street</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>displayrou</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>mi_ctrline</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>br_oneway</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>br_ow_dir</t>
+        </is>
+      </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>the_geom.type</t>
+        </is>
+      </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
+          <t>the_geom.coordinates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MARTIN LUTHER KING JR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>E 60TH ST</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>E GARFIELD BLVD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bike Lane</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.606632445511</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>[[[-87.61596722873355, 41.79447924837816], [-87.61596240494777, 41.79430050261858], [-87.61595387958901, 41.794019324842175], [-87.61595221895054, 41.793914372880195], [-87.6159492328856, 41.7937256581611], [-87.61593750022224, 41.79327162576783], [-87.61592978257218, 41.79299366364513], [-87.6159225351212, 41.79273266440588], [-87.61590789718983, 41.79214452861778], [-87.61589672766125, 41.79171566450216], [-87.61589595174317, 41.79168566437099], [-87.61588731154538, 41.791353223202755], [-87.61588373604435, 41.79116387266975], [-87.61587938048893, 41.7909332432366], [-87.61586361475077, 41.790216173130815], [-87.61584652197911, 41.78953257521417], [-87.61584193583178, 41.78934637405001], [-87.6158306194276, 41.788887047122536], [-87.61581249137379, 41.788158243893456], [-87.61579995532938, 41.78764487448411], [-87.61579650199282, 41.78751482823511], [-87.61578787016359, 41.78718979679211], [-87.61577690448134, 41.78670003809722], [-87.61575999695505, 41.78593413949687], [-87.61575383227367, 41.78569102954054]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MORGAN DR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MORGAN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>E GARFIELD BLVD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>E RAINEY DR</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.273718846564</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>[[[-87.61596722873355, 41.79447924837816], [-87.6146469845286, 41.79448424318099], [-87.61456787464198, 41.79436714347174], [-87.61450709727534, 41.79431895802028], [-87.6143985569633, 41.794255873500255], [-87.6141197215744, 41.79414946114153], [-87.61382441334366, 41.79403383425632], [-87.6134815765371, 41.79389227663244], [-87.6130801537817, 41.793723402199994], [-87.61266529980448, 41.793548871617894], [-87.61256569245539, 41.79351690629572], [-87.61228726976846, 41.793452589898784], [-87.61192237827309, 41.793381692076636], [-87.61160240422876, 41.79331461549506], [-87.61135460974891, 41.79325965395785], [-87.61113643580505, 41.79319189681021]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RAINEY DR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RAINEY</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>E MORGAN DR</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>S PAYNE DR</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.178889999619</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>[[[-87.61113643580505, 41.79319189681021], [-87.61027140525307, 41.79324090422853], [-87.60989251887229, 41.79329304690278], [-87.60937437248673, 41.79342496623983], [-87.60886325840134, 41.793616204143184], [-87.60865500686141, 41.7937165630091], [-87.60857624945564, 41.79375451664176], [-87.60832625016991, 41.793901789122955], [-87.60815780062902, 41.794007341210126], [-87.60799024123432, 41.794105496864226]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MARTIN LUTHER KING JR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>E 63RD ST</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>E 60TH ST</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Marked Shared Lane</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.376882833436</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>[[[-87.61575383227367, 41.78569102954054], [-87.61574993781109, 41.78553744521935], [-87.61574138360854, 41.78517657282576], [-87.61573776816034, 41.78502407786211], [-87.61573285074613, 41.78482393338706], [-87.61573153730231, 41.78476080670819], [-87.61572472739175, 41.78450016636337], [-87.61571872246783, 41.78427586575751], [-87.61571485138407, 41.78413637750075], [-87.61570778700545, 41.7838763432772], [-87.61569941071674, 41.78356793917766], [-87.61569566745142, 41.78337093071964], [-87.61569072742108, 41.7831267676854], [-87.6156851515035, 41.782883644180046], [-87.61568021674788, 41.78266857073254], [-87.6156740657309, 41.78240151307447], [-87.61567022077433, 41.78223337383118], [-87.615666220557, 41.78206578282973], [-87.61566197396462, 41.78188781729118], [-87.61565468608553, 41.78162077950507], [-87.61564598878145, 41.78130258011225], [-87.61563835812058, 41.78102346549074], [-87.61563106734714, 41.780756592410725], [-87.61562912474022, 41.78068679372381], [-87.61562591117682, 41.780571321066525], [-87.61562193693463, 41.78043690467687], [-87.61561662312582, 41.78023125459074]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>STONY ISLAND AVE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>STONY ISLAND</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>E 59TH ST</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>E 56TH ST</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.378464121006</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>[[[-87.58662892252528, 41.78789358129685], [-87.586706089987, 41.79153912486357], [-87.58663186923798, 41.79337593873825]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>63RD ST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>63RD</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>S MARYLAND AVE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>S STONY ISLAND AVE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Bike Lane</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.939759213128</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>[[[-87.6046422414081, 41.78042037203421], [-87.58645234642981, 41.78061152172805]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>55TH PL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>55TH</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>S DORCHESTER AVE</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>E 55TH ST</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.140520676257</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>[[[-87.59168916179809, 41.795501250471744], [-87.59156420785152, 41.79550224079574], [-87.59131454042925, 41.79550235705856], [-87.59109786212012, 41.79550386629565], [-87.59085770346485, 41.79550615703121], [-87.59063312557093, 41.79550898557082], [-87.59034113508434, 41.79551248331219], [-87.59008263205658, 41.79551557934015], [-87.58986476270361, 41.79551853261422], [-87.58969927989575, 41.795519959075364], [-87.58959813856721, 41.79551348622447], [-87.58949753203959, 41.795492500363025], [-87.58941006033334, 41.795458316572784], [-87.58930035814839, 41.79539227921674], [-87.58923659094965, 41.795287816040414], [-87.58921021181861, 41.795222275968634], [-87.58920472557244, 41.79519313923364]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>OAKWOOD BLVD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>OAKWOOD</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>S COTTAGE GROVE AVE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Bike Lane</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.521985922417</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>[[[-87.61695962339326, 41.82264134188429], [-87.61669629612875, 41.82264370313865], [-87.61606631519486, 41.822649350671306], [-87.61515537131041, 41.82265750964905], [-87.61417375753305, 41.822666282273154], [-87.61359604756068, 41.82267144039865], [-87.61289063246282, 41.82267242469886], [-87.6121351823511, 41.8226734740702], [-87.611723286215, 41.82267866256548], [-87.61021322833639, 41.82269767014164], [-87.60979638334024, 41.82270234788722], [-87.60820507512415, 41.82272019148444], [-87.6069221364619, 41.82272643226638], [-87.60684961994563, 41.822720681391324]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ELLSWORTH DR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ELLSWORTH</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>E GARFIELD BLVD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>E 51ST ST</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.563850072419</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>[[[-87.61610503358958, 41.80209463506868], [-87.61598017987416, 41.801936535122216], [-87.61571941210941, 41.80151328586742], [-87.61550944727176, 41.80119731531666], [-87.61539693942696, 41.80102858217285], [-87.61529932756855, 41.80088235809726], [-87.61506155892664, 41.80053756279236], [-87.614929442976, 41.80036126695795], [-87.6147326797903, 41.80020701596753], [-87.61447389984386, 41.800029817334064], [-87.61431845146083, 41.799919979246425], [-87.6141480647915, 41.79976531521329], [-87.61403399880841, 41.7996282102345], [-87.61398065771237, 41.799550981614956], [-87.61395599984449, 41.79950944339995], [-87.61391106290475, 41.79939892462118], [-87.61389464937568, 41.79934160352373], [-87.61388617434496, 41.799296050230076], [-87.61388737070605, 41.79922835661386], [-87.61389328726345, 41.79900113927943], [-87.61391381323126, 41.798644730896484], [-87.61392200607862, 41.79853402352384], [-87.61392355907101, 41.798501352248834], [-87.61392547720082, 41.798460992447886], [-87.61396071892041, 41.79813000580307], [-87.61400731520777, 41.79785924549823], [-87.6140570307326, 41.79763090320573], [-87.6141338608941, 41.79734899758503], [-87.61419534320311, 41.797160438942676], [-87.61428035246796, 41.79693075355048], [-87.61437410917135, 41.7966928071726], [-87.61439017940391, 41.79665131864515], [-87.61448490414, 41.79640677773468], [-87.61455078269736, 41.796175847853924], [-87.61459809192392, 41.79591974491938], [-87.61462586548868, 41.79561330073654], [-87.61463898952323, 41.7953906021651], [-87.6146621547144, 41.79508629626382], [-87.61469428955904, 41.7949442612965], [-87.61469972612767, 41.794814738076944], [-87.61469151426928, 41.79468057278534], [-87.61467818509446, 41.79459684387978], [-87.6146469845286, 41.79448424318099]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MARTIN LUTHER KING JR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>E 51ST ST</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>E 37TH ST</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1.75304400525</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>[[[-87.6170661605481, 41.82746577345483], [-87.61706142929766, 41.82722251576819], [-87.61703594211926, 41.82599621919331], [-87.6170346569476, 41.825924585756425], [-87.61702807683459, 41.825640732364505], [-87.61701815626563, 41.825212839267834], [-87.61701158986415, 41.824860489202024], [-87.61700504238831, 41.82446703021115], [-87.61699819000684, 41.82410092909017], [-87.61699111101917, 41.82382621643897], [-87.6169682780898, 41.82294010913907], [-87.61695962339326, 41.82264134188429], [-87.61694647296191, 41.82218741283243], [-87.61694134071122, 41.82200285608154], [-87.61691550518213, 41.82107381642339], [-87.61690011817095, 41.820520501742], [-87.6168912291518, 41.82022584659349], [-87.61687951834088, 41.819837625724176], [-87.61686451475447, 41.81931905960095], [-87.61685917407235, 41.819134444733976], [-87.61685486347649, 41.81903471854085], [-87.61685026940104, 41.81886108718419], [-87.61684584573, 41.818632543662474], [-87.61683899958928, 41.818426428036624], [-87.61682859667718, 41.81811322063313], [-87.61682317373558, 41.81791516029109], [-87.6168170711122, 41.81769914813044], [-87.61681204388093, 41.81752487028064], [-87.6168097679134, 41.8174459431259], [-87.61680154890371, 41.817143281582915], [-87.61680085310701, 41.81711867608355], [-87.61679454768834, 41.8168960333512], [-87.61678662778932, 41.816627119659934], [-87.61677714364522, 41.81630505574234], [-87.61677062740476, 41.81603396382891], [-87.61676552375634, 41.81582380290046], [-87.61675765682091, 41.81555209840315], [-87.61675059408309, 41.81531687029233], [-87.61674224579149, 41.815039015176694], [-87.61673544566895, 41.814814353391846], [-87.61672717933429, 41.814541247209775], [-87.61672053521322, 41.814281652787514], [-87.6167133124245, 41.814034457969235], [-87.61670518857355, 41.813756248551975], [-87.61669736056754, 41.8134778473913], [-87.61668988955066, 41.8131937690335], [-87.61668445767971, 41.813002180182174], [-87.61667472405641, 41.812658842819], [-87.616665225364, 41.812313114669124], [-87.61666403964655, 41.81227254737789], [-87.6166590672492, 41.812102152014056], [-87.61665296669604, 41.811892506022836], [-87.61664655510585, 41.811671359704654], [-87.61664207135496, 41.81149114274442], [-87.61663372407628, 41.811189079715234], [-87.61662461081087, 41.81085932970484], [-87.61662055015955, 41.81066750713534], [-87.61661158374402, 41.81035309368742], [-87.61660946369571, 41.81028007730828], [-87.61660532895206, 41.81013765741237], [-87.6165971626926, 41.809869902413276], [-87.61658969716275, 41.809631378067415], [-87.6165830260001, 41.80937622288194], [-87.61657750843742, 41.80916515967291], [-87.61657434552195, 41.80905399609861], [-87.61656977392795, 41.80889161626314], [-87.61656382612986, 41.80868147771314], [-87.6165595258573, 41.80852434140443], [-87.61655442132603, 41.80832082118215], [-87.61654832746574, 41.80807121930493], [-87.61654000442812, 41.8077846368839], [-87.61653454090984, 41.80755514196061], [-87.61652978730874, 41.80735545128697], [-87.61652116505952, 41.80702339471532], [-87.61650989769541, 41.806543569441665], [-87.6165048970603, 41.80633409577223], [-87.61649750571686, 41.805990301736024], [-87.61649069419391, 41.80573396875114], [-87.61648329413629, 41.80545551854538], [-87.6164821821902, 41.80541072451418], [-87.61647834932612, 41.8052344630603], [-87.61646633002383, 41.80475973793773], [-87.61645839638088, 41.80443169207701], [-87.61644878457702, 41.804030528954634], [-87.61644580038985, 41.803914590028064], [-87.61644156658187, 41.80375012783846], [-87.61643122120574, 41.803483868826675], [-87.61640545455953, 41.80318628304824], [-87.61636657748137, 41.803006515619764], [-87.6163590650835, 41.80297177546721], [-87.61625552696026, 41.80267897305564], [-87.61618167023049, 41.8024149789362], [-87.61610503358958, 41.80209463506868]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>55TH ST</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>55TH</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>S COTTAGE GROVE AVE</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>S DORCHESTER AVE</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.766203524173</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>[[[-87.60620979087955, 41.79495747442708], [-87.6057344224648, 41.79495778503282], [-87.60525201125915, 41.79496326297865], [-87.60479417557326, 41.794968318532064], [-87.60416578190858, 41.79497613248727], [-87.60382968914276, 41.79497974562034], [-87.60364258908545, 41.79498175626839], [-87.6031618006071, 41.79498638580917], [-87.60258003192963, 41.79499286770068], [-87.60201296951952, 41.794999330425995], [-87.60176485131475, 41.79500208669209], [-87.60130428020985, 41.79500683720651], [-87.60083389016755, 41.795011687128714], [-87.60050008922202, 41.79501581473183], [-87.6002440069741, 41.79501912014317], [-87.59977157954289, 41.79502367900555], [-87.59944937777256, 41.79502678009304], [-87.5991151755601, 41.795030737243415], [-87.59876610668249, 41.79503599750648], [-87.59846421388181, 41.795039746997446], [-87.59809252263335, 41.79504284460396], [-87.59783639943313, 41.79504497752776], [-87.59764672479376, 41.79504746882311], [-87.59746279967632, 41.79504988499188], [-87.59729500945298, 41.795051197774896], [-87.59714467615815, 41.79505237459098], [-87.59712751034556, 41.79505261932045], [-87.59653845570257, 41.79505834324881], [-87.59587785724203, 41.79506631315715], [-87.59585440739944, 41.795062984370915], [-87.59491762743127, 41.79507687701188], [-87.59334179382368, 41.795100230834926], [-87.59230182841584, 41.795115630665705], [-87.592302990093, 41.795150774423014], [-87.59230046172085, 41.795201582121706], [-87.59228243740286, 41.795250862799094], [-87.59224146498102, 41.795340996591], [-87.59222898325629, 41.79535145199423], [-87.59207943860847, 41.79544011543386], [-87.5920123125014, 41.79546698816598], [-87.59190924617853, 41.795490664939614], [-87.59181796862944, 41.7955002290602], [-87.59168916179809, 41.795501250471744]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DREXEL BLVD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DREXEL</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>E HYDE PARK BLVD</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>E OAKWOOD BLVD</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1.44027790321</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>[[[-87.6061357829986, 41.82285126887031], [-87.60609798571573, 41.82276399646166], [-87.60590091255791, 41.82238247366579], [-87.60556669332729, 41.8218485016191], [-87.60530502182334, 41.82143367779866], [-87.60503607482781, 41.82100731247258], [-87.6048651023532, 41.820736412610586], [-87.60468547053425, 41.82045272301633], [-87.60449083328942, 41.820146654278034], [-87.6044256482468, 41.820039488053965], [-87.60440298975179, 41.8199636312076], [-87.60436493891923, 41.819611683642336], [-87.60429991730739, 41.819055419679465], [-87.60429380433658, 41.81900362340333], [-87.60426189555417, 41.8187247681738], [-87.60423424833219, 41.81848098336986], [-87.60420878995686, 41.81825126419623], [-87.60417455131629, 41.817968413673675], [-87.60415552556421, 41.81781123864321], [-87.60413394449134, 41.81761153828346], [-87.60411028125793, 41.81739508449601], [-87.6040885112337, 41.8171992256062], [-87.6040700938691, 41.81703439693089], [-87.60405800489534, 41.81683774595473], [-87.60404268597567, 41.816588553468314], [-87.60403709666593, 41.81630849303128], [-87.60403120520014, 41.8160161354863], [-87.60402385839835, 41.81570661792346], [-87.6040170517352, 41.81545621443974], [-87.60400794890579, 41.81501570099713], [-87.60400263005133, 41.814758282399495], [-87.6039971166536, 41.8145069813334], [-87.60399159427311, 41.81425010973378], [-87.60398593909036, 41.81399836927459], [-87.60398044110272, 41.813765236437085], [-87.60397499985255, 41.81352699896516], [-87.60396816319397, 41.813199599950835], [-87.60396389986742, 41.8129954454885], [-87.60395896340789, 41.81276777679964], [-87.60395507075744, 41.812587068895915], [-87.60395103323813, 41.81239971908291], [-87.60394749744123, 41.81224261431615], [-87.60394634625938, 41.812192497109486], [-87.60394481883999, 41.812126322466376], [-87.60393970922209, 41.8119040592473], [-87.60393553325102, 41.81172255360749], [-87.60392887286369, 41.811376458031624], [-87.60392551762324, 41.81120206585357], [-87.6039220751111, 41.811026987049004], [-87.60391755623571, 41.81080453486339], [-87.60391271281719, 41.810565396211956], [-87.60390920747359, 41.810395859547214], [-87.60390545674095, 41.810224510714114], [-87.6039029260037, 41.810108878818895], [-87.60389805780825, 41.80989781291501], [-87.60389154426316, 41.80955704103505], [-87.60388737756344, 41.80933909368288], [-87.6038839679615, 41.80921055686321], [-87.60387961854272, 41.80904658706937], [-87.60387371153965, 41.80877837916568], [-87.60386741299754, 41.80847998089812], [-87.60386217213637, 41.80822741989517], [-87.60385829065206, 41.80802316594071], [-87.60385239269901, 41.80773868420216], [-87.60384783613233, 41.80751883906607], [-87.60384274399121, 41.807243419051346], [-87.60383646805631, 41.80693986273583], [-87.60383088501047, 41.80664640914328], [-87.6038268275711, 41.80644791716319], [-87.60381920996646, 41.8061785179137], [-87.60381478491121, 41.80591612025036], [-87.60381184231792, 41.80574166480126], [-87.60380626616268, 41.80551868439242], [-87.60380179621455, 41.80533089313059], [-87.60379613662855, 41.80512799991602], [-87.60379079943327, 41.80490019151557], [-87.6037865313686, 41.80469439808748], [-87.6037805331614, 41.80445368703591], [-87.60377677465617, 41.804267683853766], [-87.60377404877609, 41.80410075937107], [-87.60377006455334, 41.80385690535313], [-87.60376813499602, 41.80374251152941], [-87.60376478430065, 41.80361114875377], [-87.60375648729162, 41.803366141884204], [-87.60375141035728, 41.80319294589922], [-87.60374820447251, 41.803022835593254], [-87.60374626819105, 41.80289938597228], [-87.60374406398431, 41.80276709679405], [-87.603741005496, 41.802597042333126], [-87.60377786306702, 41.802278554577875]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MARTIN LUTHER KING JR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>E GARFIELD BLVD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>E 51ST ST</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Bike Lane</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.525487613949</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>[[[-87.61610503358958, 41.80209463506868], [-87.6161372553474, 41.80190169269912], [-87.61614074146709, 41.80158907436339], [-87.61612777562215, 41.80089368105505], [-87.61611061011892, 41.80022228554601], [-87.6161072447521, 41.80009063210527], [-87.61609367670414, 41.799567542526496], [-87.61608066594823, 41.799007655365806], [-87.61607252526402, 41.798655650381], [-87.61607043851457, 41.798547458174994], [-87.6160678890834, 41.798457127876596], [-87.61605837110685, 41.79805028367454], [-87.61604192712679, 41.79739045646684], [-87.6160235286314, 41.79670545121182], [-87.61602194699849, 41.79663990734271], [-87.61601550198797, 41.7963728214937], [-87.61599616418324, 41.79563948379497], [-87.61599287316523, 41.795514680599055], [-87.61597940877292, 41.795011981545464], [-87.6159753641248, 41.794792923748744], [-87.6159725954511, 41.7946429706259], [-87.61596722873355, 41.79447924837816]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>55TH ST</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>55TH</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>S HYDE PARK BLVD</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>S SHORE DR</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Marked Shared Lane</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.158892281839</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>[[[-87.58394543361024, 41.795220065764205], [-87.5835817620467, 41.795223797172596], [-87.58327948192816, 41.79522915096661], [-87.58324210928754, 41.79522947236536], [-87.5829312072739, 41.795232145317705], [-87.58253279286843, 41.79523559512813], [-87.58220685560578, 41.795238416348866], [-87.5819200476465, 41.79524101361322], [-87.58182560768654, 41.79524177247036], [-87.58163397586631, 41.79524331336056], [-87.58124686189768, 41.795246514830914], [-87.58086945340737, 41.79525705071672]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>31ST ST</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>31ST</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>S MOE DR</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.374564177222</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>[[[-87.61711743673902, 41.83841544388878], [-87.61349382112748, 41.83846417399243], [-87.61336507987872, 41.8384654324603], [-87.61170778684063, 41.8384964974145], [-87.6113260948113, 41.838513422816135], [-87.61122239818451, 41.83851802083818], [-87.61106328407865, 41.83852507577069], [-87.61079286825503, 41.83852833767229], [-87.61023646107017, 41.83853504871899], [-87.61004517815752, 41.83853385151719], [-87.60986250664294, 41.83853270823932]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>33RD ST</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>33RD</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>S STATE ST</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Marked Shared Lane</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.47034639757</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>[[[-87.62649453439884, 41.834657620039394], [-87.6261375484813, 41.834653255468275], [-87.62598820768505, 41.834655523097894], [-87.6258713558933, 41.83465729648271], [-87.62555479911322, 41.834663112644094], [-87.62521987635559, 41.834667222892755], [-87.62505539738287, 41.834670172980104], [-87.62490108129768, 41.834672941521305], [-87.62458217233613, 41.834675666707916], [-87.62423396810284, 41.83467955437231], [-87.62419467526055, 41.83468228203092], [-87.62332410153712, 41.834694699177206], [-87.6225766889668, 41.834705354550316], [-87.62204427228347, 41.83471294207457], [-87.62183407802331, 41.834710293288616], [-87.62162465056676, 41.834707653371126], [-87.62122627094816, 41.83471231672194], [-87.62080305524594, 41.834717269393636], [-87.62061503357474, 41.834712419521736], [-87.62049200866362, 41.83470924673693], [-87.6196388712932, 41.834730650392935], [-87.61940523053126, 41.834732824088015], [-87.61923746068237, 41.8347343849626], [-87.61879845501683, 41.83473992804518], [-87.61849043146212, 41.83474381686139], [-87.61818788325031, 41.83474705287812], [-87.61738398483341, 41.83475564899769]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>OAKWOOD BLVD</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>OAKWOOD</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>S COTTAGE GROVE AVE</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>E PERSHING RD</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Bike Lane</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.179532699715</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>[[[-87.60684961994563, 41.822720681391324], [-87.60679180817826, 41.82272115395717], [-87.60677001340125, 41.82272103500519], [-87.60674821900858, 41.82272120146208], [-87.60672643224186, 41.822721651572905], [-87.60670465910856, 41.822722386276055], [-87.60668290562634, 41.822723405609615], [-87.60666118024034, 41.82272470782627], [-87.60663948895807, 41.82272629386447], [-87.60661783660379, 41.82272816285434], [-87.60659623160228, 41.822730314849224], [-87.60657467999161, 41.822732748086665], [-87.60655318900317, 41.82273546171211], [-87.60653176465463, 41.82273845576364], [-87.60651041297386, 41.822741729379096], [-87.6064891412025, 41.82274528080366], [-87.60646795535817, 41.82274911007541], [-87.60644686148913, 41.82275321453169], [-87.60642586802022, 41.8227575942258], [-87.60640497858236, 41.82276224738011], [-87.60638420162077, 41.82276717224742], [-87.6063635431735, 41.82277236706532], [-87.60634300805471, 41.82277783186432], [-87.60632260352641, 41.82278356308904], [-87.60630233682008, 41.822789559885024], [-87.60628221277028, 41.82279582048222], [-87.60626223741507, 41.82280234311821], [-87.6062424168028, 41.822809125130334], [-87.60622275817514, 41.8228161647638], [-87.60620326757022, 41.822823460256195], [-87.60618394862924, 41.82283100892967], [-87.6061357829986, 41.82285126887031], [-87.60489865036251, 41.82326907790459], [-87.60488618404133, 41.823273092730936], [-87.60487521949304, 41.823276932508655], [-87.60486278852834, 41.823281650728966], [-87.60484930661205, 41.82328723021869], [-87.60483704714119, 41.823292747232735], [-87.6048271855152, 41.82329751145608], [-87.6048184078212, 41.8233020088474], [-87.60481037940755, 41.823306348027266], [-87.60480191461397, 41.82331116882633], [-87.60479333766806, 41.82331632654415], [-87.6047855007208, 41.823321295379984], [-87.6047572327323, 41.823341526083084], [-87.60471652058943, 41.82336869605984], [-87.60470052458207, 41.823382623822745], [-87.60468485482315, 41.82339675893244], [-87.60466951859557, 41.82341109603318], [-87.60465451835765, 41.823425630638965], [-87.6046398601683, 41.82344035918691], [-87.60462554648588, 41.82345527719107], [-87.60461158337955, 41.82347038018828], [-87.60459797573527, 41.82348566190726], [-87.60458472599103, 41.823501119662524], [-87.60457183902265, 41.82351674808307], [-87.60455931849212, 41.82353254269051], [-87.6045471692855, 41.82354849721349], [-87.60453539263716, 41.823564608958954], [-87.60452399584045, 41.823580871670806], [-87.60451297774297, 41.82359728084015], [-87.60450234562784, 41.82361383111117], [-87.60449210196373, 41.8236305170976], [-87.60448224799534, 41.823647335206], [-87.60447278860879, 41.823664279165065], [-87.60446372506924, 41.823681343580795], [-87.60445506224238, 41.82369852398245], [-87.6044468013934, 41.823715814976026], [-87.6044389437976, 41.82373321026731], [-87.60443149431059, 41.82375070628574], [-87.60442445419751, 41.823768297637386], [-87.6044178259476, 41.823785977135316], [-87.6044116108056, 41.823803741186076], [-87.60440581126073, 41.82382158260278], [-87.60440042855778, 41.823839497791994], [-87.60439546517577, 41.82385748046702], [-87.60439092117632, 41.823875525226285], [-87.60438680023185, 41.823893626690996], [-87.60438310121057, 41.82391177855161], [-87.60437982657116, 41.82392997632201], [-87.60437697757878, 41.82394821460817], [-87.60437455311194, 41.82396648620023], [-87.60437255682261, 41.82398478752], [-87.60437098758929, 41.824003111357584], [-87.60436926671751, 41.82403533381279], [-87.60435230548126, 41.82416287487605]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>COTTAGE GROVE AVE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>COTTAGE GROVE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>E PERSHING RD</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>E 35TH ST</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Bike Lane</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.535169697043</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>[[[-87.61062764640718, 41.83117833227938], [-87.61056121164148, 41.8309831537708], [-87.61049735143008, 41.83088969918398], [-87.61035664310229, 41.830683783743886], [-87.61021807070779, 41.83042154772161], [-87.60976457816737, 41.82954607123712], [-87.60957313929535, 41.82921206775326], [-87.60953484063897, 41.829123898452686], [-87.60947872228488, 41.82899470323354], [-87.60920191148996, 41.828461613639654], [-87.60903435707688, 41.82813505890052], [-87.60893989467102, 41.82795095517259], [-87.60881964632634, 41.82771437489353], [-87.60875245248874, 41.82758217879819], [-87.60848246060718, 41.827057116463294], [-87.60835626491398, 41.82681471429994], [-87.6082719086208, 41.82665265487381], [-87.60807609502977, 41.82626881297509], [-87.60797191429859, 41.82606348435161], [-87.6079087205916, 41.82593893804116], [-87.60784009873232, 41.82580134557496], [-87.60760573951933, 41.82534195692333], [-87.60750781352307, 41.825147209548874], [-87.6073738248817, 41.824880744701375], [-87.60728073042753, 41.82469689396191], [-87.6071500174633, 41.824439506146774], [-87.60686734794898, 41.8239569091955]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>31ST DR</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>31ST</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>S MOE DR</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>S FORT DEARBORN</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.112279352219</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>[[[-87.60986250664294, 41.83853270823932], [-87.6095086258396, 41.83853049214663], [-87.60918890021458, 41.83853812491465], [-87.60875811449299, 41.83854840731297], [-87.60865431875239, 41.83855088477592], [-87.60833750976242, 41.838558445341555], [-87.60824493561356, 41.83856065473611], [-87.60779764356145, 41.83857132811791], [-87.60768798164275, 41.83857394411922]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>OAKWOOD BLVD</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>OAKWOOD</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>E PERSHING RD</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LAKESHORE DR</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.265190300727</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>[[[-87.60435230548126, 41.82416287487605], [-87.60430631831143, 41.82416402356607], [-87.60428716161914, 41.824162095879494], [-87.60426796236939, 41.824160418216486], [-87.60424872656984, 41.824158991515496], [-87.6042294614419, 41.82415781582236], [-87.60421017058603, 41.824156892060216], [-87.60419086242726, 41.824156220282596], [-87.60417154057622, 41.82415580051237], [-87.60415221225436, 41.824155632795396], [-87.60413288226572, 41.82415571806249], [-87.60411355904553, 41.824156055466894], [-87.60409424500084, 41.824156645023855], [-87.60407494855669, 41.82415748678687], [-87.60405567333392, 41.82415857987863], [-87.60403642775758, 41.82415992435258], [-87.60401721664196, 41.82416152023936], [-87.60399804481145, 41.82416336666922], [-87.60397216606508, 41.82416626443172], [-87.60346372774372, 41.82428645007398], [-87.60283279718537, 41.82449961768677], [-87.60254227296632, 41.82459826474106], [-87.60246449645898, 41.82463065780316], [-87.60214041957721, 41.82476563187484], [-87.6020952755735, 41.8247849900892], [-87.6017964676506, 41.824913114836825], [-87.60160828555927, 41.824988222508935], [-87.60150680968545, 41.82502872373627], [-87.60091462496219, 41.825188150840695], [-87.60074975423764, 41.82519086558529], [-87.60046891563478, 41.82526537949098], [-87.60036960542857, 41.82529172834911], [-87.60027660609322, 41.82531640313449], [-87.59999145364394, 41.825392060591405], [-87.59984691458156, 41.8254304090753], [-87.5996240077739, 41.825489550046555], [-87.5995963400068, 41.82550927640572]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>31ST ST</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>31ST</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>S MICHIGAN AVE</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>S GILES AVE</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>0.204433765585</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>[[[-87.62343694336933, 41.83833704540958], [-87.62323358361407, 41.83833847406264], [-87.6219191008301, 41.838356765893344], [-87.62177979242179, 41.83835870302541], [-87.62128211303167, 41.83836481491048], [-87.62100750971918, 41.8383681865488], [-87.62063024755903, 41.83837298145963], [-87.62047048387781, 41.83837500885838], [-87.62015738391769, 41.83837922174425], [-87.61999021695806, 41.83838147080919], [-87.61947655373596, 41.838387441384285]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>35TH ST</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>35TH</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>S INDIANA AVE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Bike Lane</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>0.247640012693</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>[[[-87.62175790723948, 41.83105114677236], [-87.62147204346718, 41.83105439399251], [-87.62114680081156, 41.83105756560645], [-87.62071506301695, 41.83106177458682], [-87.62054500801808, 41.83106270827247], [-87.62038410991939, 41.83106359050268], [-87.61993842551381, 41.831068138560155], [-87.61959497831648, 41.83107164288365], [-87.61932790430228, 41.83107429835225], [-87.6192145415096, 41.83107542490796], [-87.61861331357758, 41.831080192721124], [-87.61840049624368, 41.8310834879503], [-87.61811354507196, 41.8310879292089], [-87.61794575632707, 41.83109052619566], [-87.61760482133919, 41.83109575717714], [-87.61730766754923, 41.83109415363711], [-87.61696083107093, 41.83109228088914]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>35TH ST</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>35TH</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>S STATE ST</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>S INDIANA AVE</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Marked Shared Lane</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>0.251982034456</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>[[[-87.6266385987239, 41.83100580881331], [-87.6264732958851, 41.83101107967687], [-87.62623318245583, 41.83101873668085], [-87.62601026219642, 41.831016431371204], [-87.62591536563151, 41.83101335928809], [-87.62580089456586, 41.83100965335254], [-87.62578894519758, 41.8310097769209], [-87.62528748091881, 41.83101497359384], [-87.62497040535462, 41.83101825860181], [-87.62460523369673, 41.83102204008217], [-87.62425145860854, 41.831023753331884], [-87.62423505388152, 41.83102409322796], [-87.62325146933688, 41.831035886002816], [-87.623068985482, 41.831038072800894], [-87.62257009356864, 41.831042925980455], [-87.62249985576759, 41.831043609555515], [-87.62195505561091, 41.831048907025604], [-87.62175790723948, 41.83105114677236]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PERSHING RD</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PERSHING</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>S MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>S COTTAGE GROVE AVE</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0.52273584865</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>[[[-87.61699111101917, 41.82382621643897], [-87.61672658426848, 41.823830247623874], [-87.61611742079225, 41.823839530348515], [-87.61610351380473, 41.8238397010112], [-87.6154691158385, 41.82384748030514], [-87.61514202830347, 41.82385149048068], [-87.61435832379438, 41.82386109676443], [-87.61307015328607, 41.82387688472249], [-87.61261856025574, 41.82388291330555], [-87.61213034165046, 41.82388942863265], [-87.61127647198559, 41.82389814834697], [-87.61055372981066, 41.82390552337138], [-87.60983565600785, 41.82391284582243], [-87.60958135685671, 41.82391543849396], [-87.6083907741053, 41.82392832878097], [-87.60833202655425, 41.82392896457945], [-87.60732163043673, 41.82394102449633], [-87.60702288161544, 41.823950057947265], [-87.60691033374472, 41.82395217241693], [-87.60686734794898, 41.8239569091955]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PERSHING RD</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PERSHING</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>S COTTAGE GROVE AVE</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>E OAKWOOD BLVD</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>0.135533728291</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>[[[-87.60686734794898, 41.8239569091955], [-87.60606651814183, 41.82417374136248], [-87.60576295911753, 41.82426465478336], [-87.60574292254485, 41.82427037292759], [-87.60572275653709, 41.824275828247], [-87.60570246591914, 41.82428101987172], [-87.60568205673985, 41.82428594513898], [-87.60566153743501, 41.824290603201796], [-87.60564091042225, 41.82429499317505], [-87.60562018535114, 41.824299113319164], [-87.60559936705677, 41.82430296186401], [-87.6055784615575, 41.824306538847644], [-87.60555747730946, 41.8243098416226], [-87.60553641792379, 41.8243128702117], [-87.60551529184642, 41.824315622867694], [-87.6054675496305, 41.82432080616751], [-87.60514959326278, 41.82431298815248], [-87.60506702606838, 41.82430186758017], [-87.60498473109828, 41.8242896709576], [-87.60490273359159, 41.824276402046785], [-87.60482105759388, 41.82426206370194], [-87.60473921548223, 41.8242465609951], [-87.6045999908213, 41.824210864913994], [-87.60435230548126, 41.82416287487605]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>31ST ST</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>31ST</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>S GILES AVE</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>0.121774289186</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>[[[-87.61947655373596, 41.838387441384285], [-87.61826297733084, 41.83840128373133], [-87.61746126495309, 41.838411426314124], [-87.61711743673902, 41.83841544388878]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PAYNE DR</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PAYNE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>E RAINEY DR</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>E 55TH ST</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0.0675160768248</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>[[[-87.60737728719235, 41.79496310174033], [-87.60739572258301, 41.79490141710621], [-87.60759032740498, 41.794597181214684], [-87.60781895881487, 41.79429315897816], [-87.60788597312641, 41.79420071616683], [-87.60793532745689, 41.79414594962413], [-87.60799024123432, 41.794105496864226]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>55TH PL</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>55TH</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>E 55TH ST</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>S DORCHESTER AVE</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0.0456951713071</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>[[[-87.59230182841584, 41.795115630665705], [-87.59228479651814, 41.79504607209104], [-87.59225548130618, 41.79497654411554], [-87.59219846154255, 41.79489528677071], [-87.59216267495331, 41.79487450803364], [-87.5920133591238, 41.794803290937494], [-87.59193680903836, 41.794782379617466], [-87.59185276036327, 41.794775717447465], [-87.59167067344248, 41.79477653357941]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>55TH PL</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>55TH</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>S DORCHESTER AVE</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>E 55TH ST</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0.144696496175</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>[[[-87.59167067344248, 41.79477653357941], [-87.59136866354801, 41.79477788763556], [-87.59102905319932, 41.7947802494273], [-87.5907804071988, 41.794781030192134], [-87.59057041516495, 41.79478167500291], [-87.59032230194119, 41.79478403653916], [-87.59011020296843, 41.79478605342406], [-87.58985624501801, 41.79478954209586], [-87.58964247007485, 41.794793948510694], [-87.58954419795131, 41.79480903782709], [-87.5894761210009, 41.79482602245259], [-87.5894100443973, 41.7948539709812], [-87.58930529537159, 41.794916096688844], [-87.58922782297005, 41.79504082853871], [-87.58920177375734, 41.79511475522187], [-87.58919925975736, 41.795164108872186], [-87.58920472557244, 41.79519313923364]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>55TH ST</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>55TH</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>E 55TH PL</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>S LAKE PARK AVE</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0.0858058887654</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>[[[-87.58920472557244, 41.79519313923364], [-87.58843978013414, 41.795185708334266], [-87.58754346134559, 41.795176995453275]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>55TH ST</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>55TH</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>S LAKE PARK AVE</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>S HYDE PARK BLVD</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Marked Shared Lane</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0.185855928634</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>[[[-87.58754346134559, 41.795176995453275], [-87.58738962534618, 41.795178680573635], [-87.58723653779546, 41.79518035774402], [-87.58718928018563, 41.79518087552708], [-87.587017867405, 41.79518275390326], [-87.58694172794344, 41.7951835872402], [-87.58690389104218, 41.795184002251354], [-87.58673557437942, 41.79518584540241], [-87.58671603381707, 41.795186059636485], [-87.58661850963912, 41.79518760010154], [-87.58616460134657, 41.79519476866744], [-87.58576988324349, 41.79519906136454], [-87.58540490313923, 41.795203699386356], [-87.58511445279412, 41.795207390147176], [-87.58484326462393, 41.795207078465104], [-87.58467848640464, 41.79520974297046], [-87.58451912941597, 41.795212320129835], [-87.58431745967604, 41.79521624722297], [-87.58394543361024, 41.795220065764205]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DREXEL AVE</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DREXEL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PAYNE DR</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>E HYDE PARK BLVD</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0.0259560495627</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>[[[-87.60377786306702, 41.802278554577875], [-87.60384776240414, 41.80214837273826], [-87.60390914448635, 41.80205257522945], [-87.6039959751988, 41.801940495237204]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DREXEL</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DREXEL</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>E 55TH ST</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PAYNE DR</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Marked Shared Lane</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>0.460724495671</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>[[[-87.6039959751988, 41.801940495237204], [-87.60398005001674, 41.80179839512371], [-87.60394732018125, 41.801506349931245], [-87.60394800636487, 41.801407011251754], [-87.60394177538063, 41.800830920157495], [-87.60393415361173, 41.80046182103748], [-87.60391387649038, 41.79937152781625], [-87.60389748791374, 41.798638427091994], [-87.60388128354194, 41.79789695686593], [-87.60386015715976, 41.796817882461646], [-87.60383874116336, 41.79590082721114], [-87.60382896532192, 41.795475812983724], [-87.6038116695482, 41.79541642661352], [-87.60379280282437, 41.79539201977848], [-87.60371397467722, 41.79532905985543], [-87.60367737235056, 41.795309946073175]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>55TH ST</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>55TH</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>S DREXEL AVE</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>S ELLIS AVE</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Marked Shared Lane</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>0.126909173227</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>[[[-87.60367737235056, 41.795309946073175], [-87.60363422547626, 41.79530530889886], [-87.6012208491939, 41.795333144426785]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>31ST ST</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>31ST</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>S STATE ST</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>S MICHIGAN AVE</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>0.162108043223</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>[[[-87.62657731521406, 41.83829500304858], [-87.62604576913193, 41.838301553822], [-87.62596310195929, 41.838302687863916], [-87.62571612398844, 41.83830607252936], [-87.62535872708824, 41.838309852915415], [-87.62513747761189, 41.83831347505333], [-87.62505430825347, 41.83831483673369], [-87.62467528615595, 41.83831955124879], [-87.62429216946478, 41.838326215497126], [-87.62415443007986, 41.83832770511869], [-87.62365544777839, 41.83833551099617], [-87.62343694336933, 41.83833704540958]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>INDIANA AVE</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>INDIANA</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>E GARFIELD BLVD</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>E GARFIELD BLVD</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Buffered Bike Lane</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0.0223385754247</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>[[[-87.6208315835994, 41.79439138276337], [-87.62084038953641, 41.794714985686]]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>INDIANA AVE</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>INDIANA</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>E GARFIELD BLVD</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>E 31ST ST</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Protected Bike Lane</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>3.01258704379</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>MultiLineString</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>[[[-87.62084038953641, 41.794714985686], [-87.62085281129865, 41.79522725844895], [-87.62088553211312, 41.7965073441015], [-87.62088644695537, 41.796543915816564], [-87.62092397658711, 41.79804400791659], [-87.62092040298522, 41.798191215958205], [-87.62091727595173, 41.79836556520069], [-87.62093883738828, 41.79854657799714], [-87.62096199438447, 41.799573795377476], [-87.62102112204656, 41.80201894759424], [-87.62106698675902, 41.803839766506655], [-87.62111335537706, 41.805661868259016], [-87.62115857655205, 41.807483871376355], [-87.62120718434561, 41.809303307294854], [-87.62125466765067, 41.811117100360924], [-87.62130448726721, 41.812932670214146], [-87.6213099124466, 41.81312469369885], [-87.62135313717764, 41.8147437457875], [-87.62140171476847, 41.81655610062988], [-87.62145181711834, 41.81835822286233], [-87.62150080290813, 41.82016180246785], [-87.6215515887697, 41.822008224063545], [-87.62159626319296, 41.82376737598187], [-87.62163641531164, 41.82559026112434], [-87.6216549409634, 41.82649974416645], [-87.62167588050762, 41.82740303141706], [-87.62172698340358, 41.8296165245134], [-87.62175790723948, 41.83105114677236], [-87.62179495991735, 41.832893680280165], [-87.62183407802331, 41.834710293288616], [-87.62187278204642, 41.8365029035063], [-87.62192230530282, 41.838280826193916], [-87.6219191008301, 41.838356765893344]]]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="39" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>station_name</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>short_name</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>total_docks</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>docks_in_service</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>location.type</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>location.coordinates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>a3a7a4fc-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MLK Jr Dr &amp; 47th St</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CHI00399</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>41.809851</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>-87.616279</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>[-87.616279, 41.809851]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>a3a75d8a-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>State St &amp; 35th St</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CHI00343</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>41.831036314</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>-87.6267975569</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>[-87.626797556877, 41.831036314016]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>a3ad3d08-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Prairie Ave &amp; 43rd St</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CHI00545</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>41.816658893</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-87.6194124619</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>[-87.6194124619, 41.81665889302]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>a3a9984a-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Indiana Ave &amp; 31st St</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CHI00436</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>41.838842</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-87.621857</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>[-87.621857, 41.838842]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>a3a634dd-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>State St &amp; 33rd St</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CHI00223</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>41.834734</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-87.625813</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>[-87.625813, 41.834734]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>a3ad5764-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Calumet Ave &amp; 51st St</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CHI00429</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>41.8022946509</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>-87.6180535802</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>[-87.6180535802, 41.80229465088]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>a3a640d1-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fort Dearborn Dr &amp; 31st St</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CHI00222</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>41.838556</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>-87.608218</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>[-87.608218, 41.838556]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>a3ad2d57-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>State St &amp; Pershing Rd</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CHI00491</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>41.823015238</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>-87.6265680185</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>[-87.6265680185, 41.82301523798]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1963673207600511026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wabash Ave &amp; 49th St</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CHI01987</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>41.80581</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>-87.6245</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>[-87.6245, 41.80581]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>b8c74f86-2873-4818-88ac-81d9ae374add</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Fort Dearborn Dr &amp; 31st St*</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CHI02026</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>41.838676329</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>-87.6088321209</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>[-87.608832120895, 41.838676328971]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>a3ac30c5-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cottage Grove Ave &amp; 51st St</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CHI00502</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>41.803038</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>-87.606615</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>[-87.606615, 41.803038]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>a3a97a01-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cottage Grove Ave &amp; Oakwood Blvd</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CHI00400</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>41.822985</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-87.6071</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>[-87.6071, 41.822985]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>a3a781a6-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>State St &amp; 29th St</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CHI00231</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>41.8417</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>-87.62693</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>[-87.62693, 41.8417]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>a3a743ff-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MLK Jr Dr &amp; Pershing Rd</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CHI02040</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>41.8246</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>-87.61678</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>[-87.61678, 41.8246]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>a3a859c4-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MLK Jr Dr &amp; 29th St</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CHI00386</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>41.842052</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>-87.617</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>[-87.617, 41.842052]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1963650659022207484</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>State St &amp; 45th St</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CHI02004</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>41.81313</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>-87.62585</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>[-87.62585, 41.81313]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>a3ad2843-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lake Park Ave &amp; 35th St</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CHI02032</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>41.8312742355</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>-87.6087991946</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>[-87.6087991946, 41.83127423549]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>a3a96fd5-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Rhodes Ave &amp; 32nd St</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CHI00328</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>41.836208</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>-87.613533</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>[-87.613533, 41.836208]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>a3a7aa0e-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Indiana Ave &amp; 40th St</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CHI00256</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>41.82168</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>-87.6216</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>[-87.6216, 41.82168]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>a3aae870-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cottage Grove Ave &amp; 49th St</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CHI00488</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>41.806273</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>-87.606643</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>[-87.606643, 41.806273]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>a3aae35a-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Calumet Ave &amp; 35th St</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CHI00355</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>41.831379</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>-87.618034</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>[-87.618034, 41.831379]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>a3a639f5-a135-11e9-9cda-0a87ae2ba916</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Calumet Ave &amp; 33rd St</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CHI00224</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>In Service</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>41.83472</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>-87.61797</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>[-87.61797, 41.83472]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>racktype</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>capacity</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>stands</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>41.83345</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>-87.62767</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>41.8344018</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-87.6277985</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>41.8350676</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-87.626074</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>41.8354834</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>-87.6252826</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>stands</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>41.8376861</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>-87.6274522</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>41.8386122</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-87.6278464</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>41.8388786</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-87.6252598</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>stands</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>41.8351532</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-87.6253917</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>41.8436429</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-87.6179034</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>stands</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>41.8315193</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-87.6045969</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>41.8382594</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-87.6062423</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>41.8021714</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-87.6258327</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>stands</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>41.825588</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>-87.624741</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>stands</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>41.8310116</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-87.62038</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>stands</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>41.8310276</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>-87.6185682</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bike Rack</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>rack</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>41.8314</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-87.627864</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Fix bike route rendering: handle json_normalize flattened geometry columns
The SODA API returns the_geom as a nested object, but pd.json_normalize
splits it into the_geom.type and the_geom.coordinates. Added fallback
to reconstruct the geometry dict from these flattened columns.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bronzeville_assets.xlsx
+++ b/bronzeville_assets.xlsx
@@ -12590,7 +12590,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Cottage Grove &amp; 50th Street</t>
+          <t>Canal Street railroad bridge</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -16682,12 +16682,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>STONY ISLAND AVE</t>
+          <t>55TH ST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>STONY ISLAND</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -16697,12 +16697,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>E 59TH ST</t>
+          <t>E 55TH PL</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>E 56TH ST</t>
+          <t>S LAKE PARK AVE</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -16712,7 +16712,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.378464121006</t>
+          <t>0.0858058887654</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -16732,19 +16732,19 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[[[-87.58662892252528, 41.78789358129685], [-87.586706089987, 41.79153912486357], [-87.58663186923798, 41.79337593873825]]]</t>
+          <t>[[[-87.58920472557244, 41.79519313923364], [-87.58843978013414, 41.795185708334266], [-87.58754346134559, 41.795176995453275]]]</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>63RD ST</t>
+          <t>55TH ST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>63RD</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -16754,22 +16754,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>S MARYLAND AVE</t>
+          <t>S LAKE PARK AVE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>S STONY ISLAND AVE</t>
+          <t>S HYDE PARK BLVD</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Marked Shared Lane</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.939759213128</t>
+          <t>0.185855928634</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -16789,29 +16789,29 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[[[-87.6046422414081, 41.78042037203421], [-87.58645234642981, 41.78061152172805]]]</t>
+          <t>[[[-87.58754346134559, 41.795176995453275], [-87.58738962534618, 41.795178680573635], [-87.58723653779546, 41.79518035774402], [-87.58718928018563, 41.79518087552708], [-87.587017867405, 41.79518275390326], [-87.58694172794344, 41.7951835872402], [-87.58690389104218, 41.795184002251354], [-87.58673557437942, 41.79518584540241], [-87.58671603381707, 41.795186059636485], [-87.58661850963912, 41.79518760010154], [-87.58616460134657, 41.79519476866744], [-87.58576988324349, 41.79519906136454], [-87.58540490313923, 41.795203699386356], [-87.58511445279412, 41.795207390147176], [-87.58484326462393, 41.795207078465104], [-87.58467848640464, 41.79520974297046], [-87.58451912941597, 41.795212320129835], [-87.58431745967604, 41.79521624722297], [-87.58394543361024, 41.795220065764205]]]</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>55TH PL</t>
+          <t>PAYNE DR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>PAYNE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>S DORCHESTER AVE</t>
+          <t>E RAINEY DR</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -16821,22 +16821,22 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.140520676257</t>
+          <t>0.0675160768248</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1W</t>
+          <t>2W</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -16846,54 +16846,54 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>[[[-87.59168916179809, 41.795501250471744], [-87.59156420785152, 41.79550224079574], [-87.59131454042925, 41.79550235705856], [-87.59109786212012, 41.79550386629565], [-87.59085770346485, 41.79550615703121], [-87.59063312557093, 41.79550898557082], [-87.59034113508434, 41.79551248331219], [-87.59008263205658, 41.79551557934015], [-87.58986476270361, 41.79551853261422], [-87.58969927989575, 41.795519959075364], [-87.58959813856721, 41.79551348622447], [-87.58949753203959, 41.795492500363025], [-87.58941006033334, 41.795458316572784], [-87.58930035814839, 41.79539227921674], [-87.58923659094965, 41.795287816040414], [-87.58921021181861, 41.795222275968634], [-87.58920472557244, 41.79519313923364]]]</t>
+          <t>[[[-87.60737728719235, 41.79496310174033], [-87.60739572258301, 41.79490141710621], [-87.60759032740498, 41.794597181214684], [-87.60781895881487, 41.79429315897816], [-87.60788597312641, 41.79420071616683], [-87.60793532745689, 41.79414594962413], [-87.60799024123432, 41.794105496864226]]]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>OAKWOOD BLVD</t>
+          <t>55TH PL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OAKWOOD</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>E 55TH ST</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>S COTTAGE GROVE AVE</t>
+          <t>S DORCHESTER AVE</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.521985922417</t>
+          <t>0.0456951713071</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2W</t>
+          <t>1W</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -16903,54 +16903,54 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>[[[-87.61695962339326, 41.82264134188429], [-87.61669629612875, 41.82264370313865], [-87.61606631519486, 41.822649350671306], [-87.61515537131041, 41.82265750964905], [-87.61417375753305, 41.822666282273154], [-87.61359604756068, 41.82267144039865], [-87.61289063246282, 41.82267242469886], [-87.6121351823511, 41.8226734740702], [-87.611723286215, 41.82267866256548], [-87.61021322833639, 41.82269767014164], [-87.60979638334024, 41.82270234788722], [-87.60820507512415, 41.82272019148444], [-87.6069221364619, 41.82272643226638], [-87.60684961994563, 41.822720681391324]]]</t>
+          <t>[[[-87.59230182841584, 41.795115630665705], [-87.59228479651814, 41.79504607209104], [-87.59225548130618, 41.79497654411554], [-87.59219846154255, 41.79489528677071], [-87.59216267495331, 41.79487450803364], [-87.5920133591238, 41.794803290937494], [-87.59193680903836, 41.794782379617466], [-87.59185276036327, 41.794775717447465], [-87.59167067344248, 41.79477653357941]]]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ELLSWORTH DR</t>
+          <t>55TH PL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ELLSWORTH</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>E GARFIELD BLVD</t>
+          <t>S DORCHESTER AVE</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>E 51ST ST</t>
+          <t>E 55TH ST</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.563850072419</t>
+          <t>0.144696496175</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2W</t>
+          <t>1W</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -16960,19 +16960,19 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>[[[-87.61610503358958, 41.80209463506868], [-87.61598017987416, 41.801936535122216], [-87.61571941210941, 41.80151328586742], [-87.61550944727176, 41.80119731531666], [-87.61539693942696, 41.80102858217285], [-87.61529932756855, 41.80088235809726], [-87.61506155892664, 41.80053756279236], [-87.614929442976, 41.80036126695795], [-87.6147326797903, 41.80020701596753], [-87.61447389984386, 41.800029817334064], [-87.61431845146083, 41.799919979246425], [-87.6141480647915, 41.79976531521329], [-87.61403399880841, 41.7996282102345], [-87.61398065771237, 41.799550981614956], [-87.61395599984449, 41.79950944339995], [-87.61391106290475, 41.79939892462118], [-87.61389464937568, 41.79934160352373], [-87.61388617434496, 41.799296050230076], [-87.61388737070605, 41.79922835661386], [-87.61389328726345, 41.79900113927943], [-87.61391381323126, 41.798644730896484], [-87.61392200607862, 41.79853402352384], [-87.61392355907101, 41.798501352248834], [-87.61392547720082, 41.798460992447886], [-87.61396071892041, 41.79813000580307], [-87.61400731520777, 41.79785924549823], [-87.6140570307326, 41.79763090320573], [-87.6141338608941, 41.79734899758503], [-87.61419534320311, 41.797160438942676], [-87.61428035246796, 41.79693075355048], [-87.61437410917135, 41.7966928071726], [-87.61439017940391, 41.79665131864515], [-87.61448490414, 41.79640677773468], [-87.61455078269736, 41.796175847853924], [-87.61459809192392, 41.79591974491938], [-87.61462586548868, 41.79561330073654], [-87.61463898952323, 41.7953906021651], [-87.6146621547144, 41.79508629626382], [-87.61469428955904, 41.7949442612965], [-87.61469972612767, 41.794814738076944], [-87.61469151426928, 41.79468057278534], [-87.61467818509446, 41.79459684387978], [-87.6146469845286, 41.79448424318099]]]</t>
+          <t>[[[-87.59167067344248, 41.79477653357941], [-87.59136866354801, 41.79477788763556], [-87.59102905319932, 41.7947802494273], [-87.5907804071988, 41.794781030192134], [-87.59057041516495, 41.79478167500291], [-87.59032230194119, 41.79478403653916], [-87.59011020296843, 41.79478605342406], [-87.58985624501801, 41.79478954209586], [-87.58964247007485, 41.794793948510694], [-87.58954419795131, 41.79480903782709], [-87.5894761210009, 41.79482602245259], [-87.5894100443973, 41.7948539709812], [-87.58930529537159, 41.794916096688844], [-87.58922782297005, 41.79504082853871], [-87.58920177375734, 41.79511475522187], [-87.58919925975736, 41.795164108872186], [-87.58920472557244, 41.79519313923364]]]</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MARTIN LUTHER KING JR DR</t>
+          <t>55TH ST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MARTIN LUTHER KING JR</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -16982,22 +16982,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>E 51ST ST</t>
+          <t>S HYDE PARK BLVD</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>E 37TH ST</t>
+          <t>S SHORE DR</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Marked Shared Lane</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>1.75304400525</t>
+          <t>0.158892281839</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -17017,19 +17017,19 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>[[[-87.6170661605481, 41.82746577345483], [-87.61706142929766, 41.82722251576819], [-87.61703594211926, 41.82599621919331], [-87.6170346569476, 41.825924585756425], [-87.61702807683459, 41.825640732364505], [-87.61701815626563, 41.825212839267834], [-87.61701158986415, 41.824860489202024], [-87.61700504238831, 41.82446703021115], [-87.61699819000684, 41.82410092909017], [-87.61699111101917, 41.82382621643897], [-87.6169682780898, 41.82294010913907], [-87.61695962339326, 41.82264134188429], [-87.61694647296191, 41.82218741283243], [-87.61694134071122, 41.82200285608154], [-87.61691550518213, 41.82107381642339], [-87.61690011817095, 41.820520501742], [-87.6168912291518, 41.82022584659349], [-87.61687951834088, 41.819837625724176], [-87.61686451475447, 41.81931905960095], [-87.61685917407235, 41.819134444733976], [-87.61685486347649, 41.81903471854085], [-87.61685026940104, 41.81886108718419], [-87.61684584573, 41.818632543662474], [-87.61683899958928, 41.818426428036624], [-87.61682859667718, 41.81811322063313], [-87.61682317373558, 41.81791516029109], [-87.6168170711122, 41.81769914813044], [-87.61681204388093, 41.81752487028064], [-87.6168097679134, 41.8174459431259], [-87.61680154890371, 41.817143281582915], [-87.61680085310701, 41.81711867608355], [-87.61679454768834, 41.8168960333512], [-87.61678662778932, 41.816627119659934], [-87.61677714364522, 41.81630505574234], [-87.61677062740476, 41.81603396382891], [-87.61676552375634, 41.81582380290046], [-87.61675765682091, 41.81555209840315], [-87.61675059408309, 41.81531687029233], [-87.61674224579149, 41.815039015176694], [-87.61673544566895, 41.814814353391846], [-87.61672717933429, 41.814541247209775], [-87.61672053521322, 41.814281652787514], [-87.6167133124245, 41.814034457969235], [-87.61670518857355, 41.813756248551975], [-87.61669736056754, 41.8134778473913], [-87.61668988955066, 41.8131937690335], [-87.61668445767971, 41.813002180182174], [-87.61667472405641, 41.812658842819], [-87.616665225364, 41.812313114669124], [-87.61666403964655, 41.81227254737789], [-87.6166590672492, 41.812102152014056], [-87.61665296669604, 41.811892506022836], [-87.61664655510585, 41.811671359704654], [-87.61664207135496, 41.81149114274442], [-87.61663372407628, 41.811189079715234], [-87.61662461081087, 41.81085932970484], [-87.61662055015955, 41.81066750713534], [-87.61661158374402, 41.81035309368742], [-87.61660946369571, 41.81028007730828], [-87.61660532895206, 41.81013765741237], [-87.6165971626926, 41.809869902413276], [-87.61658969716275, 41.809631378067415], [-87.6165830260001, 41.80937622288194], [-87.61657750843742, 41.80916515967291], [-87.61657434552195, 41.80905399609861], [-87.61656977392795, 41.80889161626314], [-87.61656382612986, 41.80868147771314], [-87.6165595258573, 41.80852434140443], [-87.61655442132603, 41.80832082118215], [-87.61654832746574, 41.80807121930493], [-87.61654000442812, 41.8077846368839], [-87.61653454090984, 41.80755514196061], [-87.61652978730874, 41.80735545128697], [-87.61652116505952, 41.80702339471532], [-87.61650989769541, 41.806543569441665], [-87.6165048970603, 41.80633409577223], [-87.61649750571686, 41.805990301736024], [-87.61649069419391, 41.80573396875114], [-87.61648329413629, 41.80545551854538], [-87.6164821821902, 41.80541072451418], [-87.61647834932612, 41.8052344630603], [-87.61646633002383, 41.80475973793773], [-87.61645839638088, 41.80443169207701], [-87.61644878457702, 41.804030528954634], [-87.61644580038985, 41.803914590028064], [-87.61644156658187, 41.80375012783846], [-87.61643122120574, 41.803483868826675], [-87.61640545455953, 41.80318628304824], [-87.61636657748137, 41.803006515619764], [-87.6163590650835, 41.80297177546721], [-87.61625552696026, 41.80267897305564], [-87.61618167023049, 41.8024149789362], [-87.61610503358958, 41.80209463506868]]]</t>
+          <t>[[[-87.58394543361024, 41.795220065764205], [-87.5835817620467, 41.795223797172596], [-87.58327948192816, 41.79522915096661], [-87.58324210928754, 41.79522947236536], [-87.5829312072739, 41.795232145317705], [-87.58253279286843, 41.79523559512813], [-87.58220685560578, 41.795238416348866], [-87.5819200476465, 41.79524101361322], [-87.58182560768654, 41.79524177247036], [-87.58163397586631, 41.79524331336056], [-87.58124686189768, 41.795246514830914], [-87.58086945340737, 41.79525705071672]]]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>55TH ST</t>
+          <t>STONY ISLAND AVE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>STONY ISLAND</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -17039,22 +17039,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>S COTTAGE GROVE AVE</t>
+          <t>E 59TH ST</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>S DORCHESTER AVE</t>
+          <t>E 56TH ST</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.766203524173</t>
+          <t>0.378464121006</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -17074,19 +17074,19 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>[[[-87.60620979087955, 41.79495747442708], [-87.6057344224648, 41.79495778503282], [-87.60525201125915, 41.79496326297865], [-87.60479417557326, 41.794968318532064], [-87.60416578190858, 41.79497613248727], [-87.60382968914276, 41.79497974562034], [-87.60364258908545, 41.79498175626839], [-87.6031618006071, 41.79498638580917], [-87.60258003192963, 41.79499286770068], [-87.60201296951952, 41.794999330425995], [-87.60176485131475, 41.79500208669209], [-87.60130428020985, 41.79500683720651], [-87.60083389016755, 41.795011687128714], [-87.60050008922202, 41.79501581473183], [-87.6002440069741, 41.79501912014317], [-87.59977157954289, 41.79502367900555], [-87.59944937777256, 41.79502678009304], [-87.5991151755601, 41.795030737243415], [-87.59876610668249, 41.79503599750648], [-87.59846421388181, 41.795039746997446], [-87.59809252263335, 41.79504284460396], [-87.59783639943313, 41.79504497752776], [-87.59764672479376, 41.79504746882311], [-87.59746279967632, 41.79504988499188], [-87.59729500945298, 41.795051197774896], [-87.59714467615815, 41.79505237459098], [-87.59712751034556, 41.79505261932045], [-87.59653845570257, 41.79505834324881], [-87.59587785724203, 41.79506631315715], [-87.59585440739944, 41.795062984370915], [-87.59491762743127, 41.79507687701188], [-87.59334179382368, 41.795100230834926], [-87.59230182841584, 41.795115630665705], [-87.592302990093, 41.795150774423014], [-87.59230046172085, 41.795201582121706], [-87.59228243740286, 41.795250862799094], [-87.59224146498102, 41.795340996591], [-87.59222898325629, 41.79535145199423], [-87.59207943860847, 41.79544011543386], [-87.5920123125014, 41.79546698816598], [-87.59190924617853, 41.795490664939614], [-87.59181796862944, 41.7955002290602], [-87.59168916179809, 41.795501250471744]]]</t>
+          <t>[[[-87.58662892252528, 41.78789358129685], [-87.586706089987, 41.79153912486357], [-87.58663186923798, 41.79337593873825]]]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DREXEL BLVD</t>
+          <t>63RD ST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DREXEL</t>
+          <t>63RD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -17096,22 +17096,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>E HYDE PARK BLVD</t>
+          <t>S MARYLAND AVE</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>E OAKWOOD BLVD</t>
+          <t>S STONY ISLAND AVE</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1.44027790321</t>
+          <t>0.939759213128</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -17131,54 +17131,54 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>[[[-87.6061357829986, 41.82285126887031], [-87.60609798571573, 41.82276399646166], [-87.60590091255791, 41.82238247366579], [-87.60556669332729, 41.8218485016191], [-87.60530502182334, 41.82143367779866], [-87.60503607482781, 41.82100731247258], [-87.6048651023532, 41.820736412610586], [-87.60468547053425, 41.82045272301633], [-87.60449083328942, 41.820146654278034], [-87.6044256482468, 41.820039488053965], [-87.60440298975179, 41.8199636312076], [-87.60436493891923, 41.819611683642336], [-87.60429991730739, 41.819055419679465], [-87.60429380433658, 41.81900362340333], [-87.60426189555417, 41.8187247681738], [-87.60423424833219, 41.81848098336986], [-87.60420878995686, 41.81825126419623], [-87.60417455131629, 41.817968413673675], [-87.60415552556421, 41.81781123864321], [-87.60413394449134, 41.81761153828346], [-87.60411028125793, 41.81739508449601], [-87.6040885112337, 41.8171992256062], [-87.6040700938691, 41.81703439693089], [-87.60405800489534, 41.81683774595473], [-87.60404268597567, 41.816588553468314], [-87.60403709666593, 41.81630849303128], [-87.60403120520014, 41.8160161354863], [-87.60402385839835, 41.81570661792346], [-87.6040170517352, 41.81545621443974], [-87.60400794890579, 41.81501570099713], [-87.60400263005133, 41.814758282399495], [-87.6039971166536, 41.8145069813334], [-87.60399159427311, 41.81425010973378], [-87.60398593909036, 41.81399836927459], [-87.60398044110272, 41.813765236437085], [-87.60397499985255, 41.81352699896516], [-87.60396816319397, 41.813199599950835], [-87.60396389986742, 41.8129954454885], [-87.60395896340789, 41.81276777679964], [-87.60395507075744, 41.812587068895915], [-87.60395103323813, 41.81239971908291], [-87.60394749744123, 41.81224261431615], [-87.60394634625938, 41.812192497109486], [-87.60394481883999, 41.812126322466376], [-87.60393970922209, 41.8119040592473], [-87.60393553325102, 41.81172255360749], [-87.60392887286369, 41.811376458031624], [-87.60392551762324, 41.81120206585357], [-87.6039220751111, 41.811026987049004], [-87.60391755623571, 41.81080453486339], [-87.60391271281719, 41.810565396211956], [-87.60390920747359, 41.810395859547214], [-87.60390545674095, 41.810224510714114], [-87.6039029260037, 41.810108878818895], [-87.60389805780825, 41.80989781291501], [-87.60389154426316, 41.80955704103505], [-87.60388737756344, 41.80933909368288], [-87.6038839679615, 41.80921055686321], [-87.60387961854272, 41.80904658706937], [-87.60387371153965, 41.80877837916568], [-87.60386741299754, 41.80847998089812], [-87.60386217213637, 41.80822741989517], [-87.60385829065206, 41.80802316594071], [-87.60385239269901, 41.80773868420216], [-87.60384783613233, 41.80751883906607], [-87.60384274399121, 41.807243419051346], [-87.60383646805631, 41.80693986273583], [-87.60383088501047, 41.80664640914328], [-87.6038268275711, 41.80644791716319], [-87.60381920996646, 41.8061785179137], [-87.60381478491121, 41.80591612025036], [-87.60381184231792, 41.80574166480126], [-87.60380626616268, 41.80551868439242], [-87.60380179621455, 41.80533089313059], [-87.60379613662855, 41.80512799991602], [-87.60379079943327, 41.80490019151557], [-87.6037865313686, 41.80469439808748], [-87.6037805331614, 41.80445368703591], [-87.60377677465617, 41.804267683853766], [-87.60377404877609, 41.80410075937107], [-87.60377006455334, 41.80385690535313], [-87.60376813499602, 41.80374251152941], [-87.60376478430065, 41.80361114875377], [-87.60375648729162, 41.803366141884204], [-87.60375141035728, 41.80319294589922], [-87.60374820447251, 41.803022835593254], [-87.60374626819105, 41.80289938597228], [-87.60374406398431, 41.80276709679405], [-87.603741005496, 41.802597042333126], [-87.60377786306702, 41.802278554577875]]]</t>
+          <t>[[[-87.6046422414081, 41.78042037203421], [-87.58645234642981, 41.78061152172805]]]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MARTIN LUTHER KING JR DR</t>
+          <t>55TH PL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MARTIN LUTHER KING JR</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>E GARFIELD BLVD</t>
+          <t>S DORCHESTER AVE</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>E 51ST ST</t>
+          <t>E 55TH ST</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.525487613949</t>
+          <t>0.140520676257</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2W</t>
+          <t>1W</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -17188,19 +17188,19 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>[[[-87.61610503358958, 41.80209463506868], [-87.6161372553474, 41.80190169269912], [-87.61614074146709, 41.80158907436339], [-87.61612777562215, 41.80089368105505], [-87.61611061011892, 41.80022228554601], [-87.6161072447521, 41.80009063210527], [-87.61609367670414, 41.799567542526496], [-87.61608066594823, 41.799007655365806], [-87.61607252526402, 41.798655650381], [-87.61607043851457, 41.798547458174994], [-87.6160678890834, 41.798457127876596], [-87.61605837110685, 41.79805028367454], [-87.61604192712679, 41.79739045646684], [-87.6160235286314, 41.79670545121182], [-87.61602194699849, 41.79663990734271], [-87.61601550198797, 41.7963728214937], [-87.61599616418324, 41.79563948379497], [-87.61599287316523, 41.795514680599055], [-87.61597940877292, 41.795011981545464], [-87.6159753641248, 41.794792923748744], [-87.6159725954511, 41.7946429706259], [-87.61596722873355, 41.79447924837816]]]</t>
+          <t>[[[-87.59168916179809, 41.795501250471744], [-87.59156420785152, 41.79550224079574], [-87.59131454042925, 41.79550235705856], [-87.59109786212012, 41.79550386629565], [-87.59085770346485, 41.79550615703121], [-87.59063312557093, 41.79550898557082], [-87.59034113508434, 41.79551248331219], [-87.59008263205658, 41.79551557934015], [-87.58986476270361, 41.79551853261422], [-87.58969927989575, 41.795519959075364], [-87.58959813856721, 41.79551348622447], [-87.58949753203959, 41.795492500363025], [-87.58941006033334, 41.795458316572784], [-87.58930035814839, 41.79539227921674], [-87.58923659094965, 41.795287816040414], [-87.58921021181861, 41.795222275968634], [-87.58920472557244, 41.79519313923364]]]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>55TH ST</t>
+          <t>OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>OAKWOOD</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -17210,22 +17210,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>S HYDE PARK BLVD</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>S SHORE DR</t>
+          <t>S COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Marked Shared Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.158892281839</t>
+          <t>0.521985922417</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -17245,19 +17245,19 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>[[[-87.58394543361024, 41.795220065764205], [-87.5835817620467, 41.795223797172596], [-87.58327948192816, 41.79522915096661], [-87.58324210928754, 41.79522947236536], [-87.5829312072739, 41.795232145317705], [-87.58253279286843, 41.79523559512813], [-87.58220685560578, 41.795238416348866], [-87.5819200476465, 41.79524101361322], [-87.58182560768654, 41.79524177247036], [-87.58163397586631, 41.79524331336056], [-87.58124686189768, 41.795246514830914], [-87.58086945340737, 41.79525705071672]]]</t>
+          <t>[[[-87.61695962339326, 41.82264134188429], [-87.61669629612875, 41.82264370313865], [-87.61606631519486, 41.822649350671306], [-87.61515537131041, 41.82265750964905], [-87.61417375753305, 41.822666282273154], [-87.61359604756068, 41.82267144039865], [-87.61289063246282, 41.82267242469886], [-87.6121351823511, 41.8226734740702], [-87.611723286215, 41.82267866256548], [-87.61021322833639, 41.82269767014164], [-87.60979638334024, 41.82270234788722], [-87.60820507512415, 41.82272019148444], [-87.6069221364619, 41.82272643226638], [-87.60684961994563, 41.822720681391324]]]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>31ST ST</t>
+          <t>ELLSWORTH DR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>31ST</t>
+          <t>ELLSWORTH</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -17267,12 +17267,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>E GARFIELD BLVD</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>S MOE DR</t>
+          <t>E 51ST ST</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0.374564177222</t>
+          <t>0.563850072419</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -17302,19 +17302,19 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>[[[-87.61711743673902, 41.83841544388878], [-87.61349382112748, 41.83846417399243], [-87.61336507987872, 41.8384654324603], [-87.61170778684063, 41.8384964974145], [-87.6113260948113, 41.838513422816135], [-87.61122239818451, 41.83851802083818], [-87.61106328407865, 41.83852507577069], [-87.61079286825503, 41.83852833767229], [-87.61023646107017, 41.83853504871899], [-87.61004517815752, 41.83853385151719], [-87.60986250664294, 41.83853270823932]]]</t>
+          <t>[[[-87.61610503358958, 41.80209463506868], [-87.61598017987416, 41.801936535122216], [-87.61571941210941, 41.80151328586742], [-87.61550944727176, 41.80119731531666], [-87.61539693942696, 41.80102858217285], [-87.61529932756855, 41.80088235809726], [-87.61506155892664, 41.80053756279236], [-87.614929442976, 41.80036126695795], [-87.6147326797903, 41.80020701596753], [-87.61447389984386, 41.800029817334064], [-87.61431845146083, 41.799919979246425], [-87.6141480647915, 41.79976531521329], [-87.61403399880841, 41.7996282102345], [-87.61398065771237, 41.799550981614956], [-87.61395599984449, 41.79950944339995], [-87.61391106290475, 41.79939892462118], [-87.61389464937568, 41.79934160352373], [-87.61388617434496, 41.799296050230076], [-87.61388737070605, 41.79922835661386], [-87.61389328726345, 41.79900113927943], [-87.61391381323126, 41.798644730896484], [-87.61392200607862, 41.79853402352384], [-87.61392355907101, 41.798501352248834], [-87.61392547720082, 41.798460992447886], [-87.61396071892041, 41.79813000580307], [-87.61400731520777, 41.79785924549823], [-87.6140570307326, 41.79763090320573], [-87.6141338608941, 41.79734899758503], [-87.61419534320311, 41.797160438942676], [-87.61428035246796, 41.79693075355048], [-87.61437410917135, 41.7966928071726], [-87.61439017940391, 41.79665131864515], [-87.61448490414, 41.79640677773468], [-87.61455078269736, 41.796175847853924], [-87.61459809192392, 41.79591974491938], [-87.61462586548868, 41.79561330073654], [-87.61463898952323, 41.7953906021651], [-87.6146621547144, 41.79508629626382], [-87.61469428955904, 41.7949442612965], [-87.61469972612767, 41.794814738076944], [-87.61469151426928, 41.79468057278534], [-87.61467818509446, 41.79459684387978], [-87.6146469845286, 41.79448424318099]]]</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>33RD ST</t>
+          <t>MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>33RD</t>
+          <t>MARTIN LUTHER KING JR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -17324,22 +17324,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>S STATE ST</t>
+          <t>E 51ST ST</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>E 37TH ST</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Marked Shared Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>0.47034639757</t>
+          <t>1.75304400525</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -17359,19 +17359,19 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>[[[-87.62649453439884, 41.834657620039394], [-87.6261375484813, 41.834653255468275], [-87.62598820768505, 41.834655523097894], [-87.6258713558933, 41.83465729648271], [-87.62555479911322, 41.834663112644094], [-87.62521987635559, 41.834667222892755], [-87.62505539738287, 41.834670172980104], [-87.62490108129768, 41.834672941521305], [-87.62458217233613, 41.834675666707916], [-87.62423396810284, 41.83467955437231], [-87.62419467526055, 41.83468228203092], [-87.62332410153712, 41.834694699177206], [-87.6225766889668, 41.834705354550316], [-87.62204427228347, 41.83471294207457], [-87.62183407802331, 41.834710293288616], [-87.62162465056676, 41.834707653371126], [-87.62122627094816, 41.83471231672194], [-87.62080305524594, 41.834717269393636], [-87.62061503357474, 41.834712419521736], [-87.62049200866362, 41.83470924673693], [-87.6196388712932, 41.834730650392935], [-87.61940523053126, 41.834732824088015], [-87.61923746068237, 41.8347343849626], [-87.61879845501683, 41.83473992804518], [-87.61849043146212, 41.83474381686139], [-87.61818788325031, 41.83474705287812], [-87.61738398483341, 41.83475564899769]]]</t>
+          <t>[[[-87.6170661605481, 41.82746577345483], [-87.61706142929766, 41.82722251576819], [-87.61703594211926, 41.82599621919331], [-87.6170346569476, 41.825924585756425], [-87.61702807683459, 41.825640732364505], [-87.61701815626563, 41.825212839267834], [-87.61701158986415, 41.824860489202024], [-87.61700504238831, 41.82446703021115], [-87.61699819000684, 41.82410092909017], [-87.61699111101917, 41.82382621643897], [-87.6169682780898, 41.82294010913907], [-87.61695962339326, 41.82264134188429], [-87.61694647296191, 41.82218741283243], [-87.61694134071122, 41.82200285608154], [-87.61691550518213, 41.82107381642339], [-87.61690011817095, 41.820520501742], [-87.6168912291518, 41.82022584659349], [-87.61687951834088, 41.819837625724176], [-87.61686451475447, 41.81931905960095], [-87.61685917407235, 41.819134444733976], [-87.61685486347649, 41.81903471854085], [-87.61685026940104, 41.81886108718419], [-87.61684584573, 41.818632543662474], [-87.61683899958928, 41.818426428036624], [-87.61682859667718, 41.81811322063313], [-87.61682317373558, 41.81791516029109], [-87.6168170711122, 41.81769914813044], [-87.61681204388093, 41.81752487028064], [-87.6168097679134, 41.8174459431259], [-87.61680154890371, 41.817143281582915], [-87.61680085310701, 41.81711867608355], [-87.61679454768834, 41.8168960333512], [-87.61678662778932, 41.816627119659934], [-87.61677714364522, 41.81630505574234], [-87.61677062740476, 41.81603396382891], [-87.61676552375634, 41.81582380290046], [-87.61675765682091, 41.81555209840315], [-87.61675059408309, 41.81531687029233], [-87.61674224579149, 41.815039015176694], [-87.61673544566895, 41.814814353391846], [-87.61672717933429, 41.814541247209775], [-87.61672053521322, 41.814281652787514], [-87.6167133124245, 41.814034457969235], [-87.61670518857355, 41.813756248551975], [-87.61669736056754, 41.8134778473913], [-87.61668988955066, 41.8131937690335], [-87.61668445767971, 41.813002180182174], [-87.61667472405641, 41.812658842819], [-87.616665225364, 41.812313114669124], [-87.61666403964655, 41.81227254737789], [-87.6166590672492, 41.812102152014056], [-87.61665296669604, 41.811892506022836], [-87.61664655510585, 41.811671359704654], [-87.61664207135496, 41.81149114274442], [-87.61663372407628, 41.811189079715234], [-87.61662461081087, 41.81085932970484], [-87.61662055015955, 41.81066750713534], [-87.61661158374402, 41.81035309368742], [-87.61660946369571, 41.81028007730828], [-87.61660532895206, 41.81013765741237], [-87.6165971626926, 41.809869902413276], [-87.61658969716275, 41.809631378067415], [-87.6165830260001, 41.80937622288194], [-87.61657750843742, 41.80916515967291], [-87.61657434552195, 41.80905399609861], [-87.61656977392795, 41.80889161626314], [-87.61656382612986, 41.80868147771314], [-87.6165595258573, 41.80852434140443], [-87.61655442132603, 41.80832082118215], [-87.61654832746574, 41.80807121930493], [-87.61654000442812, 41.8077846368839], [-87.61653454090984, 41.80755514196061], [-87.61652978730874, 41.80735545128697], [-87.61652116505952, 41.80702339471532], [-87.61650989769541, 41.806543569441665], [-87.6165048970603, 41.80633409577223], [-87.61649750571686, 41.805990301736024], [-87.61649069419391, 41.80573396875114], [-87.61648329413629, 41.80545551854538], [-87.6164821821902, 41.80541072451418], [-87.61647834932612, 41.8052344630603], [-87.61646633002383, 41.80475973793773], [-87.61645839638088, 41.80443169207701], [-87.61644878457702, 41.804030528954634], [-87.61644580038985, 41.803914590028064], [-87.61644156658187, 41.80375012783846], [-87.61643122120574, 41.803483868826675], [-87.61640545455953, 41.80318628304824], [-87.61636657748137, 41.803006515619764], [-87.6163590650835, 41.80297177546721], [-87.61625552696026, 41.80267897305564], [-87.61618167023049, 41.8024149789362], [-87.61610503358958, 41.80209463506868]]]</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OAKWOOD BLVD</t>
+          <t>55TH ST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OAKWOOD</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -17386,17 +17386,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>E PERSHING RD</t>
+          <t>S DORCHESTER AVE</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.179532699715</t>
+          <t>0.766203524173</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -17416,19 +17416,19 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>[[[-87.60684961994563, 41.822720681391324], [-87.60679180817826, 41.82272115395717], [-87.60677001340125, 41.82272103500519], [-87.60674821900858, 41.82272120146208], [-87.60672643224186, 41.822721651572905], [-87.60670465910856, 41.822722386276055], [-87.60668290562634, 41.822723405609615], [-87.60666118024034, 41.82272470782627], [-87.60663948895807, 41.82272629386447], [-87.60661783660379, 41.82272816285434], [-87.60659623160228, 41.822730314849224], [-87.60657467999161, 41.822732748086665], [-87.60655318900317, 41.82273546171211], [-87.60653176465463, 41.82273845576364], [-87.60651041297386, 41.822741729379096], [-87.6064891412025, 41.82274528080366], [-87.60646795535817, 41.82274911007541], [-87.60644686148913, 41.82275321453169], [-87.60642586802022, 41.8227575942258], [-87.60640497858236, 41.82276224738011], [-87.60638420162077, 41.82276717224742], [-87.6063635431735, 41.82277236706532], [-87.60634300805471, 41.82277783186432], [-87.60632260352641, 41.82278356308904], [-87.60630233682008, 41.822789559885024], [-87.60628221277028, 41.82279582048222], [-87.60626223741507, 41.82280234311821], [-87.6062424168028, 41.822809125130334], [-87.60622275817514, 41.8228161647638], [-87.60620326757022, 41.822823460256195], [-87.60618394862924, 41.82283100892967], [-87.6061357829986, 41.82285126887031], [-87.60489865036251, 41.82326907790459], [-87.60488618404133, 41.823273092730936], [-87.60487521949304, 41.823276932508655], [-87.60486278852834, 41.823281650728966], [-87.60484930661205, 41.82328723021869], [-87.60483704714119, 41.823292747232735], [-87.6048271855152, 41.82329751145608], [-87.6048184078212, 41.8233020088474], [-87.60481037940755, 41.823306348027266], [-87.60480191461397, 41.82331116882633], [-87.60479333766806, 41.82331632654415], [-87.6047855007208, 41.823321295379984], [-87.6047572327323, 41.823341526083084], [-87.60471652058943, 41.82336869605984], [-87.60470052458207, 41.823382623822745], [-87.60468485482315, 41.82339675893244], [-87.60466951859557, 41.82341109603318], [-87.60465451835765, 41.823425630638965], [-87.6046398601683, 41.82344035918691], [-87.60462554648588, 41.82345527719107], [-87.60461158337955, 41.82347038018828], [-87.60459797573527, 41.82348566190726], [-87.60458472599103, 41.823501119662524], [-87.60457183902265, 41.82351674808307], [-87.60455931849212, 41.82353254269051], [-87.6045471692855, 41.82354849721349], [-87.60453539263716, 41.823564608958954], [-87.60452399584045, 41.823580871670806], [-87.60451297774297, 41.82359728084015], [-87.60450234562784, 41.82361383111117], [-87.60449210196373, 41.8236305170976], [-87.60448224799534, 41.823647335206], [-87.60447278860879, 41.823664279165065], [-87.60446372506924, 41.823681343580795], [-87.60445506224238, 41.82369852398245], [-87.6044468013934, 41.823715814976026], [-87.6044389437976, 41.82373321026731], [-87.60443149431059, 41.82375070628574], [-87.60442445419751, 41.823768297637386], [-87.6044178259476, 41.823785977135316], [-87.6044116108056, 41.823803741186076], [-87.60440581126073, 41.82382158260278], [-87.60440042855778, 41.823839497791994], [-87.60439546517577, 41.82385748046702], [-87.60439092117632, 41.823875525226285], [-87.60438680023185, 41.823893626690996], [-87.60438310121057, 41.82391177855161], [-87.60437982657116, 41.82392997632201], [-87.60437697757878, 41.82394821460817], [-87.60437455311194, 41.82396648620023], [-87.60437255682261, 41.82398478752], [-87.60437098758929, 41.824003111357584], [-87.60436926671751, 41.82403533381279], [-87.60435230548126, 41.82416287487605]]]</t>
+          <t>[[[-87.60620979087955, 41.79495747442708], [-87.6057344224648, 41.79495778503282], [-87.60525201125915, 41.79496326297865], [-87.60479417557326, 41.794968318532064], [-87.60416578190858, 41.79497613248727], [-87.60382968914276, 41.79497974562034], [-87.60364258908545, 41.79498175626839], [-87.6031618006071, 41.79498638580917], [-87.60258003192963, 41.79499286770068], [-87.60201296951952, 41.794999330425995], [-87.60176485131475, 41.79500208669209], [-87.60130428020985, 41.79500683720651], [-87.60083389016755, 41.795011687128714], [-87.60050008922202, 41.79501581473183], [-87.6002440069741, 41.79501912014317], [-87.59977157954289, 41.79502367900555], [-87.59944937777256, 41.79502678009304], [-87.5991151755601, 41.795030737243415], [-87.59876610668249, 41.79503599750648], [-87.59846421388181, 41.795039746997446], [-87.59809252263335, 41.79504284460396], [-87.59783639943313, 41.79504497752776], [-87.59764672479376, 41.79504746882311], [-87.59746279967632, 41.79504988499188], [-87.59729500945298, 41.795051197774896], [-87.59714467615815, 41.79505237459098], [-87.59712751034556, 41.79505261932045], [-87.59653845570257, 41.79505834324881], [-87.59587785724203, 41.79506631315715], [-87.59585440739944, 41.795062984370915], [-87.59491762743127, 41.79507687701188], [-87.59334179382368, 41.795100230834926], [-87.59230182841584, 41.795115630665705], [-87.592302990093, 41.795150774423014], [-87.59230046172085, 41.795201582121706], [-87.59228243740286, 41.795250862799094], [-87.59224146498102, 41.795340996591], [-87.59222898325629, 41.79535145199423], [-87.59207943860847, 41.79544011543386], [-87.5920123125014, 41.79546698816598], [-87.59190924617853, 41.795490664939614], [-87.59181796862944, 41.7955002290602], [-87.59168916179809, 41.795501250471744]]]</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>COTTAGE GROVE AVE</t>
+          <t>DREXEL BLVD</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>COTTAGE GROVE</t>
+          <t>DREXEL</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -17438,22 +17438,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>E PERSHING RD</t>
+          <t>E HYDE PARK BLVD</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>E 35TH ST</t>
+          <t>E OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0.535169697043</t>
+          <t>1.44027790321</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -17473,19 +17473,19 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>[[[-87.61062764640718, 41.83117833227938], [-87.61056121164148, 41.8309831537708], [-87.61049735143008, 41.83088969918398], [-87.61035664310229, 41.830683783743886], [-87.61021807070779, 41.83042154772161], [-87.60976457816737, 41.82954607123712], [-87.60957313929535, 41.82921206775326], [-87.60953484063897, 41.829123898452686], [-87.60947872228488, 41.82899470323354], [-87.60920191148996, 41.828461613639654], [-87.60903435707688, 41.82813505890052], [-87.60893989467102, 41.82795095517259], [-87.60881964632634, 41.82771437489353], [-87.60875245248874, 41.82758217879819], [-87.60848246060718, 41.827057116463294], [-87.60835626491398, 41.82681471429994], [-87.6082719086208, 41.82665265487381], [-87.60807609502977, 41.82626881297509], [-87.60797191429859, 41.82606348435161], [-87.6079087205916, 41.82593893804116], [-87.60784009873232, 41.82580134557496], [-87.60760573951933, 41.82534195692333], [-87.60750781352307, 41.825147209548874], [-87.6073738248817, 41.824880744701375], [-87.60728073042753, 41.82469689396191], [-87.6071500174633, 41.824439506146774], [-87.60686734794898, 41.8239569091955]]]</t>
+          <t>[[[-87.6061357829986, 41.82285126887031], [-87.60609798571573, 41.82276399646166], [-87.60590091255791, 41.82238247366579], [-87.60556669332729, 41.8218485016191], [-87.60530502182334, 41.82143367779866], [-87.60503607482781, 41.82100731247258], [-87.6048651023532, 41.820736412610586], [-87.60468547053425, 41.82045272301633], [-87.60449083328942, 41.820146654278034], [-87.6044256482468, 41.820039488053965], [-87.60440298975179, 41.8199636312076], [-87.60436493891923, 41.819611683642336], [-87.60429991730739, 41.819055419679465], [-87.60429380433658, 41.81900362340333], [-87.60426189555417, 41.8187247681738], [-87.60423424833219, 41.81848098336986], [-87.60420878995686, 41.81825126419623], [-87.60417455131629, 41.817968413673675], [-87.60415552556421, 41.81781123864321], [-87.60413394449134, 41.81761153828346], [-87.60411028125793, 41.81739508449601], [-87.6040885112337, 41.8171992256062], [-87.6040700938691, 41.81703439693089], [-87.60405800489534, 41.81683774595473], [-87.60404268597567, 41.816588553468314], [-87.60403709666593, 41.81630849303128], [-87.60403120520014, 41.8160161354863], [-87.60402385839835, 41.81570661792346], [-87.6040170517352, 41.81545621443974], [-87.60400794890579, 41.81501570099713], [-87.60400263005133, 41.814758282399495], [-87.6039971166536, 41.8145069813334], [-87.60399159427311, 41.81425010973378], [-87.60398593909036, 41.81399836927459], [-87.60398044110272, 41.813765236437085], [-87.60397499985255, 41.81352699896516], [-87.60396816319397, 41.813199599950835], [-87.60396389986742, 41.8129954454885], [-87.60395896340789, 41.81276777679964], [-87.60395507075744, 41.812587068895915], [-87.60395103323813, 41.81239971908291], [-87.60394749744123, 41.81224261431615], [-87.60394634625938, 41.812192497109486], [-87.60394481883999, 41.812126322466376], [-87.60393970922209, 41.8119040592473], [-87.60393553325102, 41.81172255360749], [-87.60392887286369, 41.811376458031624], [-87.60392551762324, 41.81120206585357], [-87.6039220751111, 41.811026987049004], [-87.60391755623571, 41.81080453486339], [-87.60391271281719, 41.810565396211956], [-87.60390920747359, 41.810395859547214], [-87.60390545674095, 41.810224510714114], [-87.6039029260037, 41.810108878818895], [-87.60389805780825, 41.80989781291501], [-87.60389154426316, 41.80955704103505], [-87.60388737756344, 41.80933909368288], [-87.6038839679615, 41.80921055686321], [-87.60387961854272, 41.80904658706937], [-87.60387371153965, 41.80877837916568], [-87.60386741299754, 41.80847998089812], [-87.60386217213637, 41.80822741989517], [-87.60385829065206, 41.80802316594071], [-87.60385239269901, 41.80773868420216], [-87.60384783613233, 41.80751883906607], [-87.60384274399121, 41.807243419051346], [-87.60383646805631, 41.80693986273583], [-87.60383088501047, 41.80664640914328], [-87.6038268275711, 41.80644791716319], [-87.60381920996646, 41.8061785179137], [-87.60381478491121, 41.80591612025036], [-87.60381184231792, 41.80574166480126], [-87.60380626616268, 41.80551868439242], [-87.60380179621455, 41.80533089313059], [-87.60379613662855, 41.80512799991602], [-87.60379079943327, 41.80490019151557], [-87.6037865313686, 41.80469439808748], [-87.6037805331614, 41.80445368703591], [-87.60377677465617, 41.804267683853766], [-87.60377404877609, 41.80410075937107], [-87.60377006455334, 41.80385690535313], [-87.60376813499602, 41.80374251152941], [-87.60376478430065, 41.80361114875377], [-87.60375648729162, 41.803366141884204], [-87.60375141035728, 41.80319294589922], [-87.60374820447251, 41.803022835593254], [-87.60374626819105, 41.80289938597228], [-87.60374406398431, 41.80276709679405], [-87.603741005496, 41.802597042333126], [-87.60377786306702, 41.802278554577875]]]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>31ST DR</t>
+          <t>MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>31ST</t>
+          <t>MARTIN LUTHER KING JR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -17495,22 +17495,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>S MOE DR</t>
+          <t>E GARFIELD BLVD</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>S FORT DEARBORN</t>
+          <t>E 51ST ST</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0.112279352219</t>
+          <t>0.525487613949</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -17530,19 +17530,19 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>[[[-87.60986250664294, 41.83853270823932], [-87.6095086258396, 41.83853049214663], [-87.60918890021458, 41.83853812491465], [-87.60875811449299, 41.83854840731297], [-87.60865431875239, 41.83855088477592], [-87.60833750976242, 41.838558445341555], [-87.60824493561356, 41.83856065473611], [-87.60779764356145, 41.83857132811791], [-87.60768798164275, 41.83857394411922]]]</t>
+          <t>[[[-87.61610503358958, 41.80209463506868], [-87.6161372553474, 41.80190169269912], [-87.61614074146709, 41.80158907436339], [-87.61612777562215, 41.80089368105505], [-87.61611061011892, 41.80022228554601], [-87.6161072447521, 41.80009063210527], [-87.61609367670414, 41.799567542526496], [-87.61608066594823, 41.799007655365806], [-87.61607252526402, 41.798655650381], [-87.61607043851457, 41.798547458174994], [-87.6160678890834, 41.798457127876596], [-87.61605837110685, 41.79805028367454], [-87.61604192712679, 41.79739045646684], [-87.6160235286314, 41.79670545121182], [-87.61602194699849, 41.79663990734271], [-87.61601550198797, 41.7963728214937], [-87.61599616418324, 41.79563948379497], [-87.61599287316523, 41.795514680599055], [-87.61597940877292, 41.795011981545464], [-87.6159753641248, 41.794792923748744], [-87.6159725954511, 41.7946429706259], [-87.61596722873355, 41.79447924837816]]]</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OAKWOOD BLVD</t>
+          <t>31ST ST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>OAKWOOD</t>
+          <t>31ST</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -17552,22 +17552,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>E PERSHING RD</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LAKESHORE DR</t>
+          <t>S MOE DR</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.265190300727</t>
+          <t>0.374564177222</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -17587,19 +17587,19 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>[[[-87.60435230548126, 41.82416287487605], [-87.60430631831143, 41.82416402356607], [-87.60428716161914, 41.824162095879494], [-87.60426796236939, 41.824160418216486], [-87.60424872656984, 41.824158991515496], [-87.6042294614419, 41.82415781582236], [-87.60421017058603, 41.824156892060216], [-87.60419086242726, 41.824156220282596], [-87.60417154057622, 41.82415580051237], [-87.60415221225436, 41.824155632795396], [-87.60413288226572, 41.82415571806249], [-87.60411355904553, 41.824156055466894], [-87.60409424500084, 41.824156645023855], [-87.60407494855669, 41.82415748678687], [-87.60405567333392, 41.82415857987863], [-87.60403642775758, 41.82415992435258], [-87.60401721664196, 41.82416152023936], [-87.60399804481145, 41.82416336666922], [-87.60397216606508, 41.82416626443172], [-87.60346372774372, 41.82428645007398], [-87.60283279718537, 41.82449961768677], [-87.60254227296632, 41.82459826474106], [-87.60246449645898, 41.82463065780316], [-87.60214041957721, 41.82476563187484], [-87.6020952755735, 41.8247849900892], [-87.6017964676506, 41.824913114836825], [-87.60160828555927, 41.824988222508935], [-87.60150680968545, 41.82502872373627], [-87.60091462496219, 41.825188150840695], [-87.60074975423764, 41.82519086558529], [-87.60046891563478, 41.82526537949098], [-87.60036960542857, 41.82529172834911], [-87.60027660609322, 41.82531640313449], [-87.59999145364394, 41.825392060591405], [-87.59984691458156, 41.8254304090753], [-87.5996240077739, 41.825489550046555], [-87.5995963400068, 41.82550927640572]]]</t>
+          <t>[[[-87.61711743673902, 41.83841544388878], [-87.61349382112748, 41.83846417399243], [-87.61336507987872, 41.8384654324603], [-87.61170778684063, 41.8384964974145], [-87.6113260948113, 41.838513422816135], [-87.61122239818451, 41.83851802083818], [-87.61106328407865, 41.83852507577069], [-87.61079286825503, 41.83852833767229], [-87.61023646107017, 41.83853504871899], [-87.61004517815752, 41.83853385151719], [-87.60986250664294, 41.83853270823932]]]</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>31ST ST</t>
+          <t>33RD ST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>31ST</t>
+          <t>33RD</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -17609,22 +17609,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>S MICHIGAN AVE</t>
+          <t>S STATE ST</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>S GILES AVE</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Marked Shared Lane</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0.204433765585</t>
+          <t>0.47034639757</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -17644,19 +17644,19 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>[[[-87.62343694336933, 41.83833704540958], [-87.62323358361407, 41.83833847406264], [-87.6219191008301, 41.838356765893344], [-87.62177979242179, 41.83835870302541], [-87.62128211303167, 41.83836481491048], [-87.62100750971918, 41.8383681865488], [-87.62063024755903, 41.83837298145963], [-87.62047048387781, 41.83837500885838], [-87.62015738391769, 41.83837922174425], [-87.61999021695806, 41.83838147080919], [-87.61947655373596, 41.838387441384285]]]</t>
+          <t>[[[-87.62649453439884, 41.834657620039394], [-87.6261375484813, 41.834653255468275], [-87.62598820768505, 41.834655523097894], [-87.6258713558933, 41.83465729648271], [-87.62555479911322, 41.834663112644094], [-87.62521987635559, 41.834667222892755], [-87.62505539738287, 41.834670172980104], [-87.62490108129768, 41.834672941521305], [-87.62458217233613, 41.834675666707916], [-87.62423396810284, 41.83467955437231], [-87.62419467526055, 41.83468228203092], [-87.62332410153712, 41.834694699177206], [-87.6225766889668, 41.834705354550316], [-87.62204427228347, 41.83471294207457], [-87.62183407802331, 41.834710293288616], [-87.62162465056676, 41.834707653371126], [-87.62122627094816, 41.83471231672194], [-87.62080305524594, 41.834717269393636], [-87.62061503357474, 41.834712419521736], [-87.62049200866362, 41.83470924673693], [-87.6196388712932, 41.834730650392935], [-87.61940523053126, 41.834732824088015], [-87.61923746068237, 41.8347343849626], [-87.61879845501683, 41.83473992804518], [-87.61849043146212, 41.83474381686139], [-87.61818788325031, 41.83474705287812], [-87.61738398483341, 41.83475564899769]]]</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>35TH ST</t>
+          <t>OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>35TH</t>
+          <t>OAKWOOD</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -17666,12 +17666,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>S INDIANA AVE</t>
+          <t>S COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>E PERSHING RD</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -17681,7 +17681,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.247640012693</t>
+          <t>0.179532699715</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -17701,19 +17701,19 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>[[[-87.62175790723948, 41.83105114677236], [-87.62147204346718, 41.83105439399251], [-87.62114680081156, 41.83105756560645], [-87.62071506301695, 41.83106177458682], [-87.62054500801808, 41.83106270827247], [-87.62038410991939, 41.83106359050268], [-87.61993842551381, 41.831068138560155], [-87.61959497831648, 41.83107164288365], [-87.61932790430228, 41.83107429835225], [-87.6192145415096, 41.83107542490796], [-87.61861331357758, 41.831080192721124], [-87.61840049624368, 41.8310834879503], [-87.61811354507196, 41.8310879292089], [-87.61794575632707, 41.83109052619566], [-87.61760482133919, 41.83109575717714], [-87.61730766754923, 41.83109415363711], [-87.61696083107093, 41.83109228088914]]]</t>
+          <t>[[[-87.60684961994563, 41.822720681391324], [-87.60679180817826, 41.82272115395717], [-87.60677001340125, 41.82272103500519], [-87.60674821900858, 41.82272120146208], [-87.60672643224186, 41.822721651572905], [-87.60670465910856, 41.822722386276055], [-87.60668290562634, 41.822723405609615], [-87.60666118024034, 41.82272470782627], [-87.60663948895807, 41.82272629386447], [-87.60661783660379, 41.82272816285434], [-87.60659623160228, 41.822730314849224], [-87.60657467999161, 41.822732748086665], [-87.60655318900317, 41.82273546171211], [-87.60653176465463, 41.82273845576364], [-87.60651041297386, 41.822741729379096], [-87.6064891412025, 41.82274528080366], [-87.60646795535817, 41.82274911007541], [-87.60644686148913, 41.82275321453169], [-87.60642586802022, 41.8227575942258], [-87.60640497858236, 41.82276224738011], [-87.60638420162077, 41.82276717224742], [-87.6063635431735, 41.82277236706532], [-87.60634300805471, 41.82277783186432], [-87.60632260352641, 41.82278356308904], [-87.60630233682008, 41.822789559885024], [-87.60628221277028, 41.82279582048222], [-87.60626223741507, 41.82280234311821], [-87.6062424168028, 41.822809125130334], [-87.60622275817514, 41.8228161647638], [-87.60620326757022, 41.822823460256195], [-87.60618394862924, 41.82283100892967], [-87.6061357829986, 41.82285126887031], [-87.60489865036251, 41.82326907790459], [-87.60488618404133, 41.823273092730936], [-87.60487521949304, 41.823276932508655], [-87.60486278852834, 41.823281650728966], [-87.60484930661205, 41.82328723021869], [-87.60483704714119, 41.823292747232735], [-87.6048271855152, 41.82329751145608], [-87.6048184078212, 41.8233020088474], [-87.60481037940755, 41.823306348027266], [-87.60480191461397, 41.82331116882633], [-87.60479333766806, 41.82331632654415], [-87.6047855007208, 41.823321295379984], [-87.6047572327323, 41.823341526083084], [-87.60471652058943, 41.82336869605984], [-87.60470052458207, 41.823382623822745], [-87.60468485482315, 41.82339675893244], [-87.60466951859557, 41.82341109603318], [-87.60465451835765, 41.823425630638965], [-87.6046398601683, 41.82344035918691], [-87.60462554648588, 41.82345527719107], [-87.60461158337955, 41.82347038018828], [-87.60459797573527, 41.82348566190726], [-87.60458472599103, 41.823501119662524], [-87.60457183902265, 41.82351674808307], [-87.60455931849212, 41.82353254269051], [-87.6045471692855, 41.82354849721349], [-87.60453539263716, 41.823564608958954], [-87.60452399584045, 41.823580871670806], [-87.60451297774297, 41.82359728084015], [-87.60450234562784, 41.82361383111117], [-87.60449210196373, 41.8236305170976], [-87.60448224799534, 41.823647335206], [-87.60447278860879, 41.823664279165065], [-87.60446372506924, 41.823681343580795], [-87.60445506224238, 41.82369852398245], [-87.6044468013934, 41.823715814976026], [-87.6044389437976, 41.82373321026731], [-87.60443149431059, 41.82375070628574], [-87.60442445419751, 41.823768297637386], [-87.6044178259476, 41.823785977135316], [-87.6044116108056, 41.823803741186076], [-87.60440581126073, 41.82382158260278], [-87.60440042855778, 41.823839497791994], [-87.60439546517577, 41.82385748046702], [-87.60439092117632, 41.823875525226285], [-87.60438680023185, 41.823893626690996], [-87.60438310121057, 41.82391177855161], [-87.60437982657116, 41.82392997632201], [-87.60437697757878, 41.82394821460817], [-87.60437455311194, 41.82396648620023], [-87.60437255682261, 41.82398478752], [-87.60437098758929, 41.824003111357584], [-87.60436926671751, 41.82403533381279], [-87.60435230548126, 41.82416287487605]]]</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>35TH ST</t>
+          <t>COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>35TH</t>
+          <t>COTTAGE GROVE</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -17723,22 +17723,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>S STATE ST</t>
+          <t>E PERSHING RD</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>S INDIANA AVE</t>
+          <t>E 35TH ST</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Marked Shared Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0.251982034456</t>
+          <t>0.535169697043</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -17758,19 +17758,19 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>[[[-87.6266385987239, 41.83100580881331], [-87.6264732958851, 41.83101107967687], [-87.62623318245583, 41.83101873668085], [-87.62601026219642, 41.831016431371204], [-87.62591536563151, 41.83101335928809], [-87.62580089456586, 41.83100965335254], [-87.62578894519758, 41.8310097769209], [-87.62528748091881, 41.83101497359384], [-87.62497040535462, 41.83101825860181], [-87.62460523369673, 41.83102204008217], [-87.62425145860854, 41.831023753331884], [-87.62423505388152, 41.83102409322796], [-87.62325146933688, 41.831035886002816], [-87.623068985482, 41.831038072800894], [-87.62257009356864, 41.831042925980455], [-87.62249985576759, 41.831043609555515], [-87.62195505561091, 41.831048907025604], [-87.62175790723948, 41.83105114677236]]]</t>
+          <t>[[[-87.61062764640718, 41.83117833227938], [-87.61056121164148, 41.8309831537708], [-87.61049735143008, 41.83088969918398], [-87.61035664310229, 41.830683783743886], [-87.61021807070779, 41.83042154772161], [-87.60976457816737, 41.82954607123712], [-87.60957313929535, 41.82921206775326], [-87.60953484063897, 41.829123898452686], [-87.60947872228488, 41.82899470323354], [-87.60920191148996, 41.828461613639654], [-87.60903435707688, 41.82813505890052], [-87.60893989467102, 41.82795095517259], [-87.60881964632634, 41.82771437489353], [-87.60875245248874, 41.82758217879819], [-87.60848246060718, 41.827057116463294], [-87.60835626491398, 41.82681471429994], [-87.6082719086208, 41.82665265487381], [-87.60807609502977, 41.82626881297509], [-87.60797191429859, 41.82606348435161], [-87.6079087205916, 41.82593893804116], [-87.60784009873232, 41.82580134557496], [-87.60760573951933, 41.82534195692333], [-87.60750781352307, 41.825147209548874], [-87.6073738248817, 41.824880744701375], [-87.60728073042753, 41.82469689396191], [-87.6071500174633, 41.824439506146774], [-87.60686734794898, 41.8239569091955]]]</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PERSHING RD</t>
+          <t>31ST DR</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PERSHING</t>
+          <t>31ST</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -17780,22 +17780,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>S MARTIN LUTHER KING JR DR</t>
+          <t>S MOE DR</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>S COTTAGE GROVE AVE</t>
+          <t>S FORT DEARBORN</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0.52273584865</t>
+          <t>0.112279352219</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -17815,19 +17815,19 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>[[[-87.61699111101917, 41.82382621643897], [-87.61672658426848, 41.823830247623874], [-87.61611742079225, 41.823839530348515], [-87.61610351380473, 41.8238397010112], [-87.6154691158385, 41.82384748030514], [-87.61514202830347, 41.82385149048068], [-87.61435832379438, 41.82386109676443], [-87.61307015328607, 41.82387688472249], [-87.61261856025574, 41.82388291330555], [-87.61213034165046, 41.82388942863265], [-87.61127647198559, 41.82389814834697], [-87.61055372981066, 41.82390552337138], [-87.60983565600785, 41.82391284582243], [-87.60958135685671, 41.82391543849396], [-87.6083907741053, 41.82392832878097], [-87.60833202655425, 41.82392896457945], [-87.60732163043673, 41.82394102449633], [-87.60702288161544, 41.823950057947265], [-87.60691033374472, 41.82395217241693], [-87.60686734794898, 41.8239569091955]]]</t>
+          <t>[[[-87.60986250664294, 41.83853270823932], [-87.6095086258396, 41.83853049214663], [-87.60918890021458, 41.83853812491465], [-87.60875811449299, 41.83854840731297], [-87.60865431875239, 41.83855088477592], [-87.60833750976242, 41.838558445341555], [-87.60824493561356, 41.83856065473611], [-87.60779764356145, 41.83857132811791], [-87.60768798164275, 41.83857394411922]]]</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PERSHING RD</t>
+          <t>OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PERSHING</t>
+          <t>OAKWOOD</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -17837,12 +17837,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>S COTTAGE GROVE AVE</t>
+          <t>E PERSHING RD</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>E OAKWOOD BLVD</t>
+          <t>LAKESHORE DR</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -17852,7 +17852,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0.135533728291</t>
+          <t>0.265190300727</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -17872,7 +17872,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>[[[-87.60686734794898, 41.8239569091955], [-87.60606651814183, 41.82417374136248], [-87.60576295911753, 41.82426465478336], [-87.60574292254485, 41.82427037292759], [-87.60572275653709, 41.824275828247], [-87.60570246591914, 41.82428101987172], [-87.60568205673985, 41.82428594513898], [-87.60566153743501, 41.824290603201796], [-87.60564091042225, 41.82429499317505], [-87.60562018535114, 41.824299113319164], [-87.60559936705677, 41.82430296186401], [-87.6055784615575, 41.824306538847644], [-87.60555747730946, 41.8243098416226], [-87.60553641792379, 41.8243128702117], [-87.60551529184642, 41.824315622867694], [-87.6054675496305, 41.82432080616751], [-87.60514959326278, 41.82431298815248], [-87.60506702606838, 41.82430186758017], [-87.60498473109828, 41.8242896709576], [-87.60490273359159, 41.824276402046785], [-87.60482105759388, 41.82426206370194], [-87.60473921548223, 41.8242465609951], [-87.6045999908213, 41.824210864913994], [-87.60435230548126, 41.82416287487605]]]</t>
+          <t>[[[-87.60435230548126, 41.82416287487605], [-87.60430631831143, 41.82416402356607], [-87.60428716161914, 41.824162095879494], [-87.60426796236939, 41.824160418216486], [-87.60424872656984, 41.824158991515496], [-87.6042294614419, 41.82415781582236], [-87.60421017058603, 41.824156892060216], [-87.60419086242726, 41.824156220282596], [-87.60417154057622, 41.82415580051237], [-87.60415221225436, 41.824155632795396], [-87.60413288226572, 41.82415571806249], [-87.60411355904553, 41.824156055466894], [-87.60409424500084, 41.824156645023855], [-87.60407494855669, 41.82415748678687], [-87.60405567333392, 41.82415857987863], [-87.60403642775758, 41.82415992435258], [-87.60401721664196, 41.82416152023936], [-87.60399804481145, 41.82416336666922], [-87.60397216606508, 41.82416626443172], [-87.60346372774372, 41.82428645007398], [-87.60283279718537, 41.82449961768677], [-87.60254227296632, 41.82459826474106], [-87.60246449645898, 41.82463065780316], [-87.60214041957721, 41.82476563187484], [-87.6020952755735, 41.8247849900892], [-87.6017964676506, 41.824913114836825], [-87.60160828555927, 41.824988222508935], [-87.60150680968545, 41.82502872373627], [-87.60091462496219, 41.825188150840695], [-87.60074975423764, 41.82519086558529], [-87.60046891563478, 41.82526537949098], [-87.60036960542857, 41.82529172834911], [-87.60027660609322, 41.82531640313449], [-87.59999145364394, 41.825392060591405], [-87.59984691458156, 41.8254304090753], [-87.5996240077739, 41.825489550046555], [-87.5995963400068, 41.82550927640572]]]</t>
         </is>
       </c>
     </row>
@@ -17894,14 +17894,14 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
+          <t>S MICHIGAN AVE</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
           <t>S GILES AVE</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Protected Bike Lane</t>
@@ -17909,7 +17909,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0.121774289186</t>
+          <t>0.204433765585</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -17929,19 +17929,19 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>[[[-87.61947655373596, 41.838387441384285], [-87.61826297733084, 41.83840128373133], [-87.61746126495309, 41.838411426314124], [-87.61711743673902, 41.83841544388878]]]</t>
+          <t>[[[-87.62343694336933, 41.83833704540958], [-87.62323358361407, 41.83833847406264], [-87.6219191008301, 41.838356765893344], [-87.62177979242179, 41.83835870302541], [-87.62128211303167, 41.83836481491048], [-87.62100750971918, 41.8383681865488], [-87.62063024755903, 41.83837298145963], [-87.62047048387781, 41.83837500885838], [-87.62015738391769, 41.83837922174425], [-87.61999021695806, 41.83838147080919], [-87.61947655373596, 41.838387441384285]]]</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PAYNE DR</t>
+          <t>35TH ST</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PAYNE</t>
+          <t>35TH</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -17951,22 +17951,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>E RAINEY DR</t>
+          <t>S INDIANA AVE</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>E 55TH ST</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0.0675160768248</t>
+          <t>0.247640012693</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -17986,54 +17986,54 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>[[[-87.60737728719235, 41.79496310174033], [-87.60739572258301, 41.79490141710621], [-87.60759032740498, 41.794597181214684], [-87.60781895881487, 41.79429315897816], [-87.60788597312641, 41.79420071616683], [-87.60793532745689, 41.79414594962413], [-87.60799024123432, 41.794105496864226]]]</t>
+          <t>[[[-87.62175790723948, 41.83105114677236], [-87.62147204346718, 41.83105439399251], [-87.62114680081156, 41.83105756560645], [-87.62071506301695, 41.83106177458682], [-87.62054500801808, 41.83106270827247], [-87.62038410991939, 41.83106359050268], [-87.61993842551381, 41.831068138560155], [-87.61959497831648, 41.83107164288365], [-87.61932790430228, 41.83107429835225], [-87.6192145415096, 41.83107542490796], [-87.61861331357758, 41.831080192721124], [-87.61840049624368, 41.8310834879503], [-87.61811354507196, 41.8310879292089], [-87.61794575632707, 41.83109052619566], [-87.61760482133919, 41.83109575717714], [-87.61730766754923, 41.83109415363711], [-87.61696083107093, 41.83109228088914]]]</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>55TH PL</t>
+          <t>35TH ST</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>35TH</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>E 55TH ST</t>
+          <t>S STATE ST</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>S DORCHESTER AVE</t>
+          <t>S INDIANA AVE</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Marked Shared Lane</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0.0456951713071</t>
+          <t>0.251982034456</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1W</t>
+          <t>2W</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -18043,34 +18043,34 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>[[[-87.59230182841584, 41.795115630665705], [-87.59228479651814, 41.79504607209104], [-87.59225548130618, 41.79497654411554], [-87.59219846154255, 41.79489528677071], [-87.59216267495331, 41.79487450803364], [-87.5920133591238, 41.794803290937494], [-87.59193680903836, 41.794782379617466], [-87.59185276036327, 41.794775717447465], [-87.59167067344248, 41.79477653357941]]]</t>
+          <t>[[[-87.6266385987239, 41.83100580881331], [-87.6264732958851, 41.83101107967687], [-87.62623318245583, 41.83101873668085], [-87.62601026219642, 41.831016431371204], [-87.62591536563151, 41.83101335928809], [-87.62580089456586, 41.83100965335254], [-87.62578894519758, 41.8310097769209], [-87.62528748091881, 41.83101497359384], [-87.62497040535462, 41.83101825860181], [-87.62460523369673, 41.83102204008217], [-87.62425145860854, 41.831023753331884], [-87.62423505388152, 41.83102409322796], [-87.62325146933688, 41.831035886002816], [-87.623068985482, 41.831038072800894], [-87.62257009356864, 41.831042925980455], [-87.62249985576759, 41.831043609555515], [-87.62195505561091, 41.831048907025604], [-87.62175790723948, 41.83105114677236]]]</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>55TH PL</t>
+          <t>PERSHING RD</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>PERSHING</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>S DORCHESTER AVE</t>
+          <t>S MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>E 55TH ST</t>
+          <t>S COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -18080,17 +18080,17 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.144696496175</t>
+          <t>0.52273584865</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1W</t>
+          <t>2W</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -18100,19 +18100,19 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>[[[-87.59167067344248, 41.79477653357941], [-87.59136866354801, 41.79477788763556], [-87.59102905319932, 41.7947802494273], [-87.5907804071988, 41.794781030192134], [-87.59057041516495, 41.79478167500291], [-87.59032230194119, 41.79478403653916], [-87.59011020296843, 41.79478605342406], [-87.58985624501801, 41.79478954209586], [-87.58964247007485, 41.794793948510694], [-87.58954419795131, 41.79480903782709], [-87.5894761210009, 41.79482602245259], [-87.5894100443973, 41.7948539709812], [-87.58930529537159, 41.794916096688844], [-87.58922782297005, 41.79504082853871], [-87.58920177375734, 41.79511475522187], [-87.58919925975736, 41.795164108872186], [-87.58920472557244, 41.79519313923364]]]</t>
+          <t>[[[-87.61699111101917, 41.82382621643897], [-87.61672658426848, 41.823830247623874], [-87.61611742079225, 41.823839530348515], [-87.61610351380473, 41.8238397010112], [-87.6154691158385, 41.82384748030514], [-87.61514202830347, 41.82385149048068], [-87.61435832379438, 41.82386109676443], [-87.61307015328607, 41.82387688472249], [-87.61261856025574, 41.82388291330555], [-87.61213034165046, 41.82388942863265], [-87.61127647198559, 41.82389814834697], [-87.61055372981066, 41.82390552337138], [-87.60983565600785, 41.82391284582243], [-87.60958135685671, 41.82391543849396], [-87.6083907741053, 41.82392832878097], [-87.60833202655425, 41.82392896457945], [-87.60732163043673, 41.82394102449633], [-87.60702288161544, 41.823950057947265], [-87.60691033374472, 41.82395217241693], [-87.60686734794898, 41.8239569091955]]]</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>55TH ST</t>
+          <t>PERSHING RD</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>PERSHING</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -18122,12 +18122,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>E 55TH PL</t>
+          <t>S COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>S LAKE PARK AVE</t>
+          <t>E OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -18137,7 +18137,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0.0858058887654</t>
+          <t>0.135533728291</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -18157,19 +18157,19 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>[[[-87.58920472557244, 41.79519313923364], [-87.58843978013414, 41.795185708334266], [-87.58754346134559, 41.795176995453275]]]</t>
+          <t>[[[-87.60686734794898, 41.8239569091955], [-87.60606651814183, 41.82417374136248], [-87.60576295911753, 41.82426465478336], [-87.60574292254485, 41.82427037292759], [-87.60572275653709, 41.824275828247], [-87.60570246591914, 41.82428101987172], [-87.60568205673985, 41.82428594513898], [-87.60566153743501, 41.824290603201796], [-87.60564091042225, 41.82429499317505], [-87.60562018535114, 41.824299113319164], [-87.60559936705677, 41.82430296186401], [-87.6055784615575, 41.824306538847644], [-87.60555747730946, 41.8243098416226], [-87.60553641792379, 41.8243128702117], [-87.60551529184642, 41.824315622867694], [-87.6054675496305, 41.82432080616751], [-87.60514959326278, 41.82431298815248], [-87.60506702606838, 41.82430186758017], [-87.60498473109828, 41.8242896709576], [-87.60490273359159, 41.824276402046785], [-87.60482105759388, 41.82426206370194], [-87.60473921548223, 41.8242465609951], [-87.6045999908213, 41.824210864913994], [-87.60435230548126, 41.82416287487605]]]</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>55TH ST</t>
+          <t>31ST ST</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>31ST</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -18179,22 +18179,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>S LAKE PARK AVE</t>
+          <t>S GILES AVE</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>S HYDE PARK BLVD</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Marked Shared Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0.185855928634</t>
+          <t>0.121774289186</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -18214,7 +18214,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>[[[-87.58754346134559, 41.795176995453275], [-87.58738962534618, 41.795178680573635], [-87.58723653779546, 41.79518035774402], [-87.58718928018563, 41.79518087552708], [-87.587017867405, 41.79518275390326], [-87.58694172794344, 41.7951835872402], [-87.58690389104218, 41.795184002251354], [-87.58673557437942, 41.79518584540241], [-87.58671603381707, 41.795186059636485], [-87.58661850963912, 41.79518760010154], [-87.58616460134657, 41.79519476866744], [-87.58576988324349, 41.79519906136454], [-87.58540490313923, 41.795203699386356], [-87.58511445279412, 41.795207390147176], [-87.58484326462393, 41.795207078465104], [-87.58467848640464, 41.79520974297046], [-87.58451912941597, 41.795212320129835], [-87.58431745967604, 41.79521624722297], [-87.58394543361024, 41.795220065764205]]]</t>
+          <t>[[[-87.61947655373596, 41.838387441384285], [-87.61826297733084, 41.83840128373133], [-87.61746126495309, 41.838411426314124], [-87.61711743673902, 41.83841544388878]]]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add City of Chicago Vacant Building Registry as primary vacant data source
- Parse 2,489 addresses from the Vacant Building Registry PDF (PyPDF2)
- Geocode via Census batch geocoder (99.96% hit rate)
- Handle MLK Jr Dr line-wrap edge case in PDF text extraction
- 29 new unique vacant_registered records inside Bronzeville boundary
- Dedup by proximity (~30m) prefers registry data over Cook County assessor
- New dark brown markers for City Registry entries on the map
- Updated legend with three vacant sub-types

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bronzeville_assets.xlsx
+++ b/bronzeville_assets.xlsx
@@ -16682,12 +16682,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>55TH ST</t>
+          <t>STONY ISLAND AVE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>STONY ISLAND</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -16697,12 +16697,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>E 55TH PL</t>
+          <t>E 59TH ST</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>S LAKE PARK AVE</t>
+          <t>E 56TH ST</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -16712,7 +16712,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.0858058887654</t>
+          <t>0.378464121006</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -16732,19 +16732,19 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[[[-87.58920472557244, 41.79519313923364], [-87.58843978013414, 41.795185708334266], [-87.58754346134559, 41.795176995453275]]]</t>
+          <t>[[[-87.58662892252528, 41.78789358129685], [-87.586706089987, 41.79153912486357], [-87.58663186923798, 41.79337593873825]]]</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>55TH ST</t>
+          <t>63RD ST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>63RD</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -16754,22 +16754,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>S LAKE PARK AVE</t>
+          <t>S MARYLAND AVE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>S HYDE PARK BLVD</t>
+          <t>S STONY ISLAND AVE</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Marked Shared Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.185855928634</t>
+          <t>0.939759213128</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -16789,29 +16789,29 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[[[-87.58754346134559, 41.795176995453275], [-87.58738962534618, 41.795178680573635], [-87.58723653779546, 41.79518035774402], [-87.58718928018563, 41.79518087552708], [-87.587017867405, 41.79518275390326], [-87.58694172794344, 41.7951835872402], [-87.58690389104218, 41.795184002251354], [-87.58673557437942, 41.79518584540241], [-87.58671603381707, 41.795186059636485], [-87.58661850963912, 41.79518760010154], [-87.58616460134657, 41.79519476866744], [-87.58576988324349, 41.79519906136454], [-87.58540490313923, 41.795203699386356], [-87.58511445279412, 41.795207390147176], [-87.58484326462393, 41.795207078465104], [-87.58467848640464, 41.79520974297046], [-87.58451912941597, 41.795212320129835], [-87.58431745967604, 41.79521624722297], [-87.58394543361024, 41.795220065764205]]]</t>
+          <t>[[[-87.6046422414081, 41.78042037203421], [-87.58645234642981, 41.78061152172805]]]</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PAYNE DR</t>
+          <t>55TH PL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PAYNE</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>E RAINEY DR</t>
+          <t>S DORCHESTER AVE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -16821,22 +16821,22 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.0675160768248</t>
+          <t>0.140520676257</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2W</t>
+          <t>1W</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -16846,54 +16846,54 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>[[[-87.60737728719235, 41.79496310174033], [-87.60739572258301, 41.79490141710621], [-87.60759032740498, 41.794597181214684], [-87.60781895881487, 41.79429315897816], [-87.60788597312641, 41.79420071616683], [-87.60793532745689, 41.79414594962413], [-87.60799024123432, 41.794105496864226]]]</t>
+          <t>[[[-87.59168916179809, 41.795501250471744], [-87.59156420785152, 41.79550224079574], [-87.59131454042925, 41.79550235705856], [-87.59109786212012, 41.79550386629565], [-87.59085770346485, 41.79550615703121], [-87.59063312557093, 41.79550898557082], [-87.59034113508434, 41.79551248331219], [-87.59008263205658, 41.79551557934015], [-87.58986476270361, 41.79551853261422], [-87.58969927989575, 41.795519959075364], [-87.58959813856721, 41.79551348622447], [-87.58949753203959, 41.795492500363025], [-87.58941006033334, 41.795458316572784], [-87.58930035814839, 41.79539227921674], [-87.58923659094965, 41.795287816040414], [-87.58921021181861, 41.795222275968634], [-87.58920472557244, 41.79519313923364]]]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>55TH PL</t>
+          <t>OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>OAKWOOD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>E 55TH ST</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>S DORCHESTER AVE</t>
+          <t>S COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.0456951713071</t>
+          <t>0.521985922417</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1W</t>
+          <t>2W</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -16903,54 +16903,54 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>[[[-87.59230182841584, 41.795115630665705], [-87.59228479651814, 41.79504607209104], [-87.59225548130618, 41.79497654411554], [-87.59219846154255, 41.79489528677071], [-87.59216267495331, 41.79487450803364], [-87.5920133591238, 41.794803290937494], [-87.59193680903836, 41.794782379617466], [-87.59185276036327, 41.794775717447465], [-87.59167067344248, 41.79477653357941]]]</t>
+          <t>[[[-87.61695962339326, 41.82264134188429], [-87.61669629612875, 41.82264370313865], [-87.61606631519486, 41.822649350671306], [-87.61515537131041, 41.82265750964905], [-87.61417375753305, 41.822666282273154], [-87.61359604756068, 41.82267144039865], [-87.61289063246282, 41.82267242469886], [-87.6121351823511, 41.8226734740702], [-87.611723286215, 41.82267866256548], [-87.61021322833639, 41.82269767014164], [-87.60979638334024, 41.82270234788722], [-87.60820507512415, 41.82272019148444], [-87.6069221364619, 41.82272643226638], [-87.60684961994563, 41.822720681391324]]]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>55TH PL</t>
+          <t>ELLSWORTH DR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>ELLSWORTH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>S DORCHESTER AVE</t>
+          <t>E GARFIELD BLVD</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>E 55TH ST</t>
+          <t>E 51ST ST</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.144696496175</t>
+          <t>0.563850072419</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1W</t>
+          <t>2W</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -16960,19 +16960,19 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>[[[-87.59167067344248, 41.79477653357941], [-87.59136866354801, 41.79477788763556], [-87.59102905319932, 41.7947802494273], [-87.5907804071988, 41.794781030192134], [-87.59057041516495, 41.79478167500291], [-87.59032230194119, 41.79478403653916], [-87.59011020296843, 41.79478605342406], [-87.58985624501801, 41.79478954209586], [-87.58964247007485, 41.794793948510694], [-87.58954419795131, 41.79480903782709], [-87.5894761210009, 41.79482602245259], [-87.5894100443973, 41.7948539709812], [-87.58930529537159, 41.794916096688844], [-87.58922782297005, 41.79504082853871], [-87.58920177375734, 41.79511475522187], [-87.58919925975736, 41.795164108872186], [-87.58920472557244, 41.79519313923364]]]</t>
+          <t>[[[-87.61610503358958, 41.80209463506868], [-87.61598017987416, 41.801936535122216], [-87.61571941210941, 41.80151328586742], [-87.61550944727176, 41.80119731531666], [-87.61539693942696, 41.80102858217285], [-87.61529932756855, 41.80088235809726], [-87.61506155892664, 41.80053756279236], [-87.614929442976, 41.80036126695795], [-87.6147326797903, 41.80020701596753], [-87.61447389984386, 41.800029817334064], [-87.61431845146083, 41.799919979246425], [-87.6141480647915, 41.79976531521329], [-87.61403399880841, 41.7996282102345], [-87.61398065771237, 41.799550981614956], [-87.61395599984449, 41.79950944339995], [-87.61391106290475, 41.79939892462118], [-87.61389464937568, 41.79934160352373], [-87.61388617434496, 41.799296050230076], [-87.61388737070605, 41.79922835661386], [-87.61389328726345, 41.79900113927943], [-87.61391381323126, 41.798644730896484], [-87.61392200607862, 41.79853402352384], [-87.61392355907101, 41.798501352248834], [-87.61392547720082, 41.798460992447886], [-87.61396071892041, 41.79813000580307], [-87.61400731520777, 41.79785924549823], [-87.6140570307326, 41.79763090320573], [-87.6141338608941, 41.79734899758503], [-87.61419534320311, 41.797160438942676], [-87.61428035246796, 41.79693075355048], [-87.61437410917135, 41.7966928071726], [-87.61439017940391, 41.79665131864515], [-87.61448490414, 41.79640677773468], [-87.61455078269736, 41.796175847853924], [-87.61459809192392, 41.79591974491938], [-87.61462586548868, 41.79561330073654], [-87.61463898952323, 41.7953906021651], [-87.6146621547144, 41.79508629626382], [-87.61469428955904, 41.7949442612965], [-87.61469972612767, 41.794814738076944], [-87.61469151426928, 41.79468057278534], [-87.61467818509446, 41.79459684387978], [-87.6146469845286, 41.79448424318099]]]</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>55TH ST</t>
+          <t>MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>MARTIN LUTHER KING JR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -16982,22 +16982,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>S HYDE PARK BLVD</t>
+          <t>E 51ST ST</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>S SHORE DR</t>
+          <t>E 37TH ST</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Marked Shared Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.158892281839</t>
+          <t>1.75304400525</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -17017,19 +17017,19 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>[[[-87.58394543361024, 41.795220065764205], [-87.5835817620467, 41.795223797172596], [-87.58327948192816, 41.79522915096661], [-87.58324210928754, 41.79522947236536], [-87.5829312072739, 41.795232145317705], [-87.58253279286843, 41.79523559512813], [-87.58220685560578, 41.795238416348866], [-87.5819200476465, 41.79524101361322], [-87.58182560768654, 41.79524177247036], [-87.58163397586631, 41.79524331336056], [-87.58124686189768, 41.795246514830914], [-87.58086945340737, 41.79525705071672]]]</t>
+          <t>[[[-87.6170661605481, 41.82746577345483], [-87.61706142929766, 41.82722251576819], [-87.61703594211926, 41.82599621919331], [-87.6170346569476, 41.825924585756425], [-87.61702807683459, 41.825640732364505], [-87.61701815626563, 41.825212839267834], [-87.61701158986415, 41.824860489202024], [-87.61700504238831, 41.82446703021115], [-87.61699819000684, 41.82410092909017], [-87.61699111101917, 41.82382621643897], [-87.6169682780898, 41.82294010913907], [-87.61695962339326, 41.82264134188429], [-87.61694647296191, 41.82218741283243], [-87.61694134071122, 41.82200285608154], [-87.61691550518213, 41.82107381642339], [-87.61690011817095, 41.820520501742], [-87.6168912291518, 41.82022584659349], [-87.61687951834088, 41.819837625724176], [-87.61686451475447, 41.81931905960095], [-87.61685917407235, 41.819134444733976], [-87.61685486347649, 41.81903471854085], [-87.61685026940104, 41.81886108718419], [-87.61684584573, 41.818632543662474], [-87.61683899958928, 41.818426428036624], [-87.61682859667718, 41.81811322063313], [-87.61682317373558, 41.81791516029109], [-87.6168170711122, 41.81769914813044], [-87.61681204388093, 41.81752487028064], [-87.6168097679134, 41.8174459431259], [-87.61680154890371, 41.817143281582915], [-87.61680085310701, 41.81711867608355], [-87.61679454768834, 41.8168960333512], [-87.61678662778932, 41.816627119659934], [-87.61677714364522, 41.81630505574234], [-87.61677062740476, 41.81603396382891], [-87.61676552375634, 41.81582380290046], [-87.61675765682091, 41.81555209840315], [-87.61675059408309, 41.81531687029233], [-87.61674224579149, 41.815039015176694], [-87.61673544566895, 41.814814353391846], [-87.61672717933429, 41.814541247209775], [-87.61672053521322, 41.814281652787514], [-87.6167133124245, 41.814034457969235], [-87.61670518857355, 41.813756248551975], [-87.61669736056754, 41.8134778473913], [-87.61668988955066, 41.8131937690335], [-87.61668445767971, 41.813002180182174], [-87.61667472405641, 41.812658842819], [-87.616665225364, 41.812313114669124], [-87.61666403964655, 41.81227254737789], [-87.6166590672492, 41.812102152014056], [-87.61665296669604, 41.811892506022836], [-87.61664655510585, 41.811671359704654], [-87.61664207135496, 41.81149114274442], [-87.61663372407628, 41.811189079715234], [-87.61662461081087, 41.81085932970484], [-87.61662055015955, 41.81066750713534], [-87.61661158374402, 41.81035309368742], [-87.61660946369571, 41.81028007730828], [-87.61660532895206, 41.81013765741237], [-87.6165971626926, 41.809869902413276], [-87.61658969716275, 41.809631378067415], [-87.6165830260001, 41.80937622288194], [-87.61657750843742, 41.80916515967291], [-87.61657434552195, 41.80905399609861], [-87.61656977392795, 41.80889161626314], [-87.61656382612986, 41.80868147771314], [-87.6165595258573, 41.80852434140443], [-87.61655442132603, 41.80832082118215], [-87.61654832746574, 41.80807121930493], [-87.61654000442812, 41.8077846368839], [-87.61653454090984, 41.80755514196061], [-87.61652978730874, 41.80735545128697], [-87.61652116505952, 41.80702339471532], [-87.61650989769541, 41.806543569441665], [-87.6165048970603, 41.80633409577223], [-87.61649750571686, 41.805990301736024], [-87.61649069419391, 41.80573396875114], [-87.61648329413629, 41.80545551854538], [-87.6164821821902, 41.80541072451418], [-87.61647834932612, 41.8052344630603], [-87.61646633002383, 41.80475973793773], [-87.61645839638088, 41.80443169207701], [-87.61644878457702, 41.804030528954634], [-87.61644580038985, 41.803914590028064], [-87.61644156658187, 41.80375012783846], [-87.61643122120574, 41.803483868826675], [-87.61640545455953, 41.80318628304824], [-87.61636657748137, 41.803006515619764], [-87.6163590650835, 41.80297177546721], [-87.61625552696026, 41.80267897305564], [-87.61618167023049, 41.8024149789362], [-87.61610503358958, 41.80209463506868]]]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>STONY ISLAND AVE</t>
+          <t>55TH ST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>STONY ISLAND</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -17039,22 +17039,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>E 59TH ST</t>
+          <t>S COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>E 56TH ST</t>
+          <t>S DORCHESTER AVE</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.378464121006</t>
+          <t>0.766203524173</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -17074,19 +17074,19 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>[[[-87.58662892252528, 41.78789358129685], [-87.586706089987, 41.79153912486357], [-87.58663186923798, 41.79337593873825]]]</t>
+          <t>[[[-87.60620979087955, 41.79495747442708], [-87.6057344224648, 41.79495778503282], [-87.60525201125915, 41.79496326297865], [-87.60479417557326, 41.794968318532064], [-87.60416578190858, 41.79497613248727], [-87.60382968914276, 41.79497974562034], [-87.60364258908545, 41.79498175626839], [-87.6031618006071, 41.79498638580917], [-87.60258003192963, 41.79499286770068], [-87.60201296951952, 41.794999330425995], [-87.60176485131475, 41.79500208669209], [-87.60130428020985, 41.79500683720651], [-87.60083389016755, 41.795011687128714], [-87.60050008922202, 41.79501581473183], [-87.6002440069741, 41.79501912014317], [-87.59977157954289, 41.79502367900555], [-87.59944937777256, 41.79502678009304], [-87.5991151755601, 41.795030737243415], [-87.59876610668249, 41.79503599750648], [-87.59846421388181, 41.795039746997446], [-87.59809252263335, 41.79504284460396], [-87.59783639943313, 41.79504497752776], [-87.59764672479376, 41.79504746882311], [-87.59746279967632, 41.79504988499188], [-87.59729500945298, 41.795051197774896], [-87.59714467615815, 41.79505237459098], [-87.59712751034556, 41.79505261932045], [-87.59653845570257, 41.79505834324881], [-87.59587785724203, 41.79506631315715], [-87.59585440739944, 41.795062984370915], [-87.59491762743127, 41.79507687701188], [-87.59334179382368, 41.795100230834926], [-87.59230182841584, 41.795115630665705], [-87.592302990093, 41.795150774423014], [-87.59230046172085, 41.795201582121706], [-87.59228243740286, 41.795250862799094], [-87.59224146498102, 41.795340996591], [-87.59222898325629, 41.79535145199423], [-87.59207943860847, 41.79544011543386], [-87.5920123125014, 41.79546698816598], [-87.59190924617853, 41.795490664939614], [-87.59181796862944, 41.7955002290602], [-87.59168916179809, 41.795501250471744]]]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>63RD ST</t>
+          <t>DREXEL BLVD</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>63RD</t>
+          <t>DREXEL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -17096,22 +17096,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>S MARYLAND AVE</t>
+          <t>E HYDE PARK BLVD</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>S STONY ISLAND AVE</t>
+          <t>E OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.939759213128</t>
+          <t>1.44027790321</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -17131,54 +17131,54 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>[[[-87.6046422414081, 41.78042037203421], [-87.58645234642981, 41.78061152172805]]]</t>
+          <t>[[[-87.6061357829986, 41.82285126887031], [-87.60609798571573, 41.82276399646166], [-87.60590091255791, 41.82238247366579], [-87.60556669332729, 41.8218485016191], [-87.60530502182334, 41.82143367779866], [-87.60503607482781, 41.82100731247258], [-87.6048651023532, 41.820736412610586], [-87.60468547053425, 41.82045272301633], [-87.60449083328942, 41.820146654278034], [-87.6044256482468, 41.820039488053965], [-87.60440298975179, 41.8199636312076], [-87.60436493891923, 41.819611683642336], [-87.60429991730739, 41.819055419679465], [-87.60429380433658, 41.81900362340333], [-87.60426189555417, 41.8187247681738], [-87.60423424833219, 41.81848098336986], [-87.60420878995686, 41.81825126419623], [-87.60417455131629, 41.817968413673675], [-87.60415552556421, 41.81781123864321], [-87.60413394449134, 41.81761153828346], [-87.60411028125793, 41.81739508449601], [-87.6040885112337, 41.8171992256062], [-87.6040700938691, 41.81703439693089], [-87.60405800489534, 41.81683774595473], [-87.60404268597567, 41.816588553468314], [-87.60403709666593, 41.81630849303128], [-87.60403120520014, 41.8160161354863], [-87.60402385839835, 41.81570661792346], [-87.6040170517352, 41.81545621443974], [-87.60400794890579, 41.81501570099713], [-87.60400263005133, 41.814758282399495], [-87.6039971166536, 41.8145069813334], [-87.60399159427311, 41.81425010973378], [-87.60398593909036, 41.81399836927459], [-87.60398044110272, 41.813765236437085], [-87.60397499985255, 41.81352699896516], [-87.60396816319397, 41.813199599950835], [-87.60396389986742, 41.8129954454885], [-87.60395896340789, 41.81276777679964], [-87.60395507075744, 41.812587068895915], [-87.60395103323813, 41.81239971908291], [-87.60394749744123, 41.81224261431615], [-87.60394634625938, 41.812192497109486], [-87.60394481883999, 41.812126322466376], [-87.60393970922209, 41.8119040592473], [-87.60393553325102, 41.81172255360749], [-87.60392887286369, 41.811376458031624], [-87.60392551762324, 41.81120206585357], [-87.6039220751111, 41.811026987049004], [-87.60391755623571, 41.81080453486339], [-87.60391271281719, 41.810565396211956], [-87.60390920747359, 41.810395859547214], [-87.60390545674095, 41.810224510714114], [-87.6039029260037, 41.810108878818895], [-87.60389805780825, 41.80989781291501], [-87.60389154426316, 41.80955704103505], [-87.60388737756344, 41.80933909368288], [-87.6038839679615, 41.80921055686321], [-87.60387961854272, 41.80904658706937], [-87.60387371153965, 41.80877837916568], [-87.60386741299754, 41.80847998089812], [-87.60386217213637, 41.80822741989517], [-87.60385829065206, 41.80802316594071], [-87.60385239269901, 41.80773868420216], [-87.60384783613233, 41.80751883906607], [-87.60384274399121, 41.807243419051346], [-87.60383646805631, 41.80693986273583], [-87.60383088501047, 41.80664640914328], [-87.6038268275711, 41.80644791716319], [-87.60381920996646, 41.8061785179137], [-87.60381478491121, 41.80591612025036], [-87.60381184231792, 41.80574166480126], [-87.60380626616268, 41.80551868439242], [-87.60380179621455, 41.80533089313059], [-87.60379613662855, 41.80512799991602], [-87.60379079943327, 41.80490019151557], [-87.6037865313686, 41.80469439808748], [-87.6037805331614, 41.80445368703591], [-87.60377677465617, 41.804267683853766], [-87.60377404877609, 41.80410075937107], [-87.60377006455334, 41.80385690535313], [-87.60376813499602, 41.80374251152941], [-87.60376478430065, 41.80361114875377], [-87.60375648729162, 41.803366141884204], [-87.60375141035728, 41.80319294589922], [-87.60374820447251, 41.803022835593254], [-87.60374626819105, 41.80289938597228], [-87.60374406398431, 41.80276709679405], [-87.603741005496, 41.802597042333126], [-87.60377786306702, 41.802278554577875]]]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>55TH PL</t>
+          <t>MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>MARTIN LUTHER KING JR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>S DORCHESTER AVE</t>
+          <t>E GARFIELD BLVD</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>E 55TH ST</t>
+          <t>E 51ST ST</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.140520676257</t>
+          <t>0.525487613949</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1W</t>
+          <t>2W</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -17188,19 +17188,19 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>[[[-87.59168916179809, 41.795501250471744], [-87.59156420785152, 41.79550224079574], [-87.59131454042925, 41.79550235705856], [-87.59109786212012, 41.79550386629565], [-87.59085770346485, 41.79550615703121], [-87.59063312557093, 41.79550898557082], [-87.59034113508434, 41.79551248331219], [-87.59008263205658, 41.79551557934015], [-87.58986476270361, 41.79551853261422], [-87.58969927989575, 41.795519959075364], [-87.58959813856721, 41.79551348622447], [-87.58949753203959, 41.795492500363025], [-87.58941006033334, 41.795458316572784], [-87.58930035814839, 41.79539227921674], [-87.58923659094965, 41.795287816040414], [-87.58921021181861, 41.795222275968634], [-87.58920472557244, 41.79519313923364]]]</t>
+          <t>[[[-87.61610503358958, 41.80209463506868], [-87.6161372553474, 41.80190169269912], [-87.61614074146709, 41.80158907436339], [-87.61612777562215, 41.80089368105505], [-87.61611061011892, 41.80022228554601], [-87.6161072447521, 41.80009063210527], [-87.61609367670414, 41.799567542526496], [-87.61608066594823, 41.799007655365806], [-87.61607252526402, 41.798655650381], [-87.61607043851457, 41.798547458174994], [-87.6160678890834, 41.798457127876596], [-87.61605837110685, 41.79805028367454], [-87.61604192712679, 41.79739045646684], [-87.6160235286314, 41.79670545121182], [-87.61602194699849, 41.79663990734271], [-87.61601550198797, 41.7963728214937], [-87.61599616418324, 41.79563948379497], [-87.61599287316523, 41.795514680599055], [-87.61597940877292, 41.795011981545464], [-87.6159753641248, 41.794792923748744], [-87.6159725954511, 41.7946429706259], [-87.61596722873355, 41.79447924837816]]]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OAKWOOD BLVD</t>
+          <t>55TH ST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OAKWOOD</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -17210,22 +17210,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>S HYDE PARK BLVD</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>S COTTAGE GROVE AVE</t>
+          <t>S SHORE DR</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Marked Shared Lane</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.521985922417</t>
+          <t>0.158892281839</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -17245,19 +17245,19 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>[[[-87.61695962339326, 41.82264134188429], [-87.61669629612875, 41.82264370313865], [-87.61606631519486, 41.822649350671306], [-87.61515537131041, 41.82265750964905], [-87.61417375753305, 41.822666282273154], [-87.61359604756068, 41.82267144039865], [-87.61289063246282, 41.82267242469886], [-87.6121351823511, 41.8226734740702], [-87.611723286215, 41.82267866256548], [-87.61021322833639, 41.82269767014164], [-87.60979638334024, 41.82270234788722], [-87.60820507512415, 41.82272019148444], [-87.6069221364619, 41.82272643226638], [-87.60684961994563, 41.822720681391324]]]</t>
+          <t>[[[-87.58394543361024, 41.795220065764205], [-87.5835817620467, 41.795223797172596], [-87.58327948192816, 41.79522915096661], [-87.58324210928754, 41.79522947236536], [-87.5829312072739, 41.795232145317705], [-87.58253279286843, 41.79523559512813], [-87.58220685560578, 41.795238416348866], [-87.5819200476465, 41.79524101361322], [-87.58182560768654, 41.79524177247036], [-87.58163397586631, 41.79524331336056], [-87.58124686189768, 41.795246514830914], [-87.58086945340737, 41.79525705071672]]]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ELLSWORTH DR</t>
+          <t>31ST ST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ELLSWORTH</t>
+          <t>31ST</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -17267,12 +17267,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>E GARFIELD BLVD</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>E 51ST ST</t>
+          <t>S MOE DR</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0.563850072419</t>
+          <t>0.374564177222</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -17302,19 +17302,19 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>[[[-87.61610503358958, 41.80209463506868], [-87.61598017987416, 41.801936535122216], [-87.61571941210941, 41.80151328586742], [-87.61550944727176, 41.80119731531666], [-87.61539693942696, 41.80102858217285], [-87.61529932756855, 41.80088235809726], [-87.61506155892664, 41.80053756279236], [-87.614929442976, 41.80036126695795], [-87.6147326797903, 41.80020701596753], [-87.61447389984386, 41.800029817334064], [-87.61431845146083, 41.799919979246425], [-87.6141480647915, 41.79976531521329], [-87.61403399880841, 41.7996282102345], [-87.61398065771237, 41.799550981614956], [-87.61395599984449, 41.79950944339995], [-87.61391106290475, 41.79939892462118], [-87.61389464937568, 41.79934160352373], [-87.61388617434496, 41.799296050230076], [-87.61388737070605, 41.79922835661386], [-87.61389328726345, 41.79900113927943], [-87.61391381323126, 41.798644730896484], [-87.61392200607862, 41.79853402352384], [-87.61392355907101, 41.798501352248834], [-87.61392547720082, 41.798460992447886], [-87.61396071892041, 41.79813000580307], [-87.61400731520777, 41.79785924549823], [-87.6140570307326, 41.79763090320573], [-87.6141338608941, 41.79734899758503], [-87.61419534320311, 41.797160438942676], [-87.61428035246796, 41.79693075355048], [-87.61437410917135, 41.7966928071726], [-87.61439017940391, 41.79665131864515], [-87.61448490414, 41.79640677773468], [-87.61455078269736, 41.796175847853924], [-87.61459809192392, 41.79591974491938], [-87.61462586548868, 41.79561330073654], [-87.61463898952323, 41.7953906021651], [-87.6146621547144, 41.79508629626382], [-87.61469428955904, 41.7949442612965], [-87.61469972612767, 41.794814738076944], [-87.61469151426928, 41.79468057278534], [-87.61467818509446, 41.79459684387978], [-87.6146469845286, 41.79448424318099]]]</t>
+          <t>[[[-87.61711743673902, 41.83841544388878], [-87.61349382112748, 41.83846417399243], [-87.61336507987872, 41.8384654324603], [-87.61170778684063, 41.8384964974145], [-87.6113260948113, 41.838513422816135], [-87.61122239818451, 41.83851802083818], [-87.61106328407865, 41.83852507577069], [-87.61079286825503, 41.83852833767229], [-87.61023646107017, 41.83853504871899], [-87.61004517815752, 41.83853385151719], [-87.60986250664294, 41.83853270823932]]]</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MARTIN LUTHER KING JR DR</t>
+          <t>33RD ST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MARTIN LUTHER KING JR</t>
+          <t>33RD</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -17324,22 +17324,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>E 51ST ST</t>
+          <t>S STATE ST</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>E 37TH ST</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Marked Shared Lane</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>1.75304400525</t>
+          <t>0.47034639757</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -17359,19 +17359,19 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>[[[-87.6170661605481, 41.82746577345483], [-87.61706142929766, 41.82722251576819], [-87.61703594211926, 41.82599621919331], [-87.6170346569476, 41.825924585756425], [-87.61702807683459, 41.825640732364505], [-87.61701815626563, 41.825212839267834], [-87.61701158986415, 41.824860489202024], [-87.61700504238831, 41.82446703021115], [-87.61699819000684, 41.82410092909017], [-87.61699111101917, 41.82382621643897], [-87.6169682780898, 41.82294010913907], [-87.61695962339326, 41.82264134188429], [-87.61694647296191, 41.82218741283243], [-87.61694134071122, 41.82200285608154], [-87.61691550518213, 41.82107381642339], [-87.61690011817095, 41.820520501742], [-87.6168912291518, 41.82022584659349], [-87.61687951834088, 41.819837625724176], [-87.61686451475447, 41.81931905960095], [-87.61685917407235, 41.819134444733976], [-87.61685486347649, 41.81903471854085], [-87.61685026940104, 41.81886108718419], [-87.61684584573, 41.818632543662474], [-87.61683899958928, 41.818426428036624], [-87.61682859667718, 41.81811322063313], [-87.61682317373558, 41.81791516029109], [-87.6168170711122, 41.81769914813044], [-87.61681204388093, 41.81752487028064], [-87.6168097679134, 41.8174459431259], [-87.61680154890371, 41.817143281582915], [-87.61680085310701, 41.81711867608355], [-87.61679454768834, 41.8168960333512], [-87.61678662778932, 41.816627119659934], [-87.61677714364522, 41.81630505574234], [-87.61677062740476, 41.81603396382891], [-87.61676552375634, 41.81582380290046], [-87.61675765682091, 41.81555209840315], [-87.61675059408309, 41.81531687029233], [-87.61674224579149, 41.815039015176694], [-87.61673544566895, 41.814814353391846], [-87.61672717933429, 41.814541247209775], [-87.61672053521322, 41.814281652787514], [-87.6167133124245, 41.814034457969235], [-87.61670518857355, 41.813756248551975], [-87.61669736056754, 41.8134778473913], [-87.61668988955066, 41.8131937690335], [-87.61668445767971, 41.813002180182174], [-87.61667472405641, 41.812658842819], [-87.616665225364, 41.812313114669124], [-87.61666403964655, 41.81227254737789], [-87.6166590672492, 41.812102152014056], [-87.61665296669604, 41.811892506022836], [-87.61664655510585, 41.811671359704654], [-87.61664207135496, 41.81149114274442], [-87.61663372407628, 41.811189079715234], [-87.61662461081087, 41.81085932970484], [-87.61662055015955, 41.81066750713534], [-87.61661158374402, 41.81035309368742], [-87.61660946369571, 41.81028007730828], [-87.61660532895206, 41.81013765741237], [-87.6165971626926, 41.809869902413276], [-87.61658969716275, 41.809631378067415], [-87.6165830260001, 41.80937622288194], [-87.61657750843742, 41.80916515967291], [-87.61657434552195, 41.80905399609861], [-87.61656977392795, 41.80889161626314], [-87.61656382612986, 41.80868147771314], [-87.6165595258573, 41.80852434140443], [-87.61655442132603, 41.80832082118215], [-87.61654832746574, 41.80807121930493], [-87.61654000442812, 41.8077846368839], [-87.61653454090984, 41.80755514196061], [-87.61652978730874, 41.80735545128697], [-87.61652116505952, 41.80702339471532], [-87.61650989769541, 41.806543569441665], [-87.6165048970603, 41.80633409577223], [-87.61649750571686, 41.805990301736024], [-87.61649069419391, 41.80573396875114], [-87.61648329413629, 41.80545551854538], [-87.6164821821902, 41.80541072451418], [-87.61647834932612, 41.8052344630603], [-87.61646633002383, 41.80475973793773], [-87.61645839638088, 41.80443169207701], [-87.61644878457702, 41.804030528954634], [-87.61644580038985, 41.803914590028064], [-87.61644156658187, 41.80375012783846], [-87.61643122120574, 41.803483868826675], [-87.61640545455953, 41.80318628304824], [-87.61636657748137, 41.803006515619764], [-87.6163590650835, 41.80297177546721], [-87.61625552696026, 41.80267897305564], [-87.61618167023049, 41.8024149789362], [-87.61610503358958, 41.80209463506868]]]</t>
+          <t>[[[-87.62649453439884, 41.834657620039394], [-87.6261375484813, 41.834653255468275], [-87.62598820768505, 41.834655523097894], [-87.6258713558933, 41.83465729648271], [-87.62555479911322, 41.834663112644094], [-87.62521987635559, 41.834667222892755], [-87.62505539738287, 41.834670172980104], [-87.62490108129768, 41.834672941521305], [-87.62458217233613, 41.834675666707916], [-87.62423396810284, 41.83467955437231], [-87.62419467526055, 41.83468228203092], [-87.62332410153712, 41.834694699177206], [-87.6225766889668, 41.834705354550316], [-87.62204427228347, 41.83471294207457], [-87.62183407802331, 41.834710293288616], [-87.62162465056676, 41.834707653371126], [-87.62122627094816, 41.83471231672194], [-87.62080305524594, 41.834717269393636], [-87.62061503357474, 41.834712419521736], [-87.62049200866362, 41.83470924673693], [-87.6196388712932, 41.834730650392935], [-87.61940523053126, 41.834732824088015], [-87.61923746068237, 41.8347343849626], [-87.61879845501683, 41.83473992804518], [-87.61849043146212, 41.83474381686139], [-87.61818788325031, 41.83474705287812], [-87.61738398483341, 41.83475564899769]]]</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>55TH ST</t>
+          <t>OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>55TH</t>
+          <t>OAKWOOD</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -17386,17 +17386,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>S DORCHESTER AVE</t>
+          <t>E PERSHING RD</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.766203524173</t>
+          <t>0.179532699715</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -17416,19 +17416,19 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>[[[-87.60620979087955, 41.79495747442708], [-87.6057344224648, 41.79495778503282], [-87.60525201125915, 41.79496326297865], [-87.60479417557326, 41.794968318532064], [-87.60416578190858, 41.79497613248727], [-87.60382968914276, 41.79497974562034], [-87.60364258908545, 41.79498175626839], [-87.6031618006071, 41.79498638580917], [-87.60258003192963, 41.79499286770068], [-87.60201296951952, 41.794999330425995], [-87.60176485131475, 41.79500208669209], [-87.60130428020985, 41.79500683720651], [-87.60083389016755, 41.795011687128714], [-87.60050008922202, 41.79501581473183], [-87.6002440069741, 41.79501912014317], [-87.59977157954289, 41.79502367900555], [-87.59944937777256, 41.79502678009304], [-87.5991151755601, 41.795030737243415], [-87.59876610668249, 41.79503599750648], [-87.59846421388181, 41.795039746997446], [-87.59809252263335, 41.79504284460396], [-87.59783639943313, 41.79504497752776], [-87.59764672479376, 41.79504746882311], [-87.59746279967632, 41.79504988499188], [-87.59729500945298, 41.795051197774896], [-87.59714467615815, 41.79505237459098], [-87.59712751034556, 41.79505261932045], [-87.59653845570257, 41.79505834324881], [-87.59587785724203, 41.79506631315715], [-87.59585440739944, 41.795062984370915], [-87.59491762743127, 41.79507687701188], [-87.59334179382368, 41.795100230834926], [-87.59230182841584, 41.795115630665705], [-87.592302990093, 41.795150774423014], [-87.59230046172085, 41.795201582121706], [-87.59228243740286, 41.795250862799094], [-87.59224146498102, 41.795340996591], [-87.59222898325629, 41.79535145199423], [-87.59207943860847, 41.79544011543386], [-87.5920123125014, 41.79546698816598], [-87.59190924617853, 41.795490664939614], [-87.59181796862944, 41.7955002290602], [-87.59168916179809, 41.795501250471744]]]</t>
+          <t>[[[-87.60684961994563, 41.822720681391324], [-87.60679180817826, 41.82272115395717], [-87.60677001340125, 41.82272103500519], [-87.60674821900858, 41.82272120146208], [-87.60672643224186, 41.822721651572905], [-87.60670465910856, 41.822722386276055], [-87.60668290562634, 41.822723405609615], [-87.60666118024034, 41.82272470782627], [-87.60663948895807, 41.82272629386447], [-87.60661783660379, 41.82272816285434], [-87.60659623160228, 41.822730314849224], [-87.60657467999161, 41.822732748086665], [-87.60655318900317, 41.82273546171211], [-87.60653176465463, 41.82273845576364], [-87.60651041297386, 41.822741729379096], [-87.6064891412025, 41.82274528080366], [-87.60646795535817, 41.82274911007541], [-87.60644686148913, 41.82275321453169], [-87.60642586802022, 41.8227575942258], [-87.60640497858236, 41.82276224738011], [-87.60638420162077, 41.82276717224742], [-87.6063635431735, 41.82277236706532], [-87.60634300805471, 41.82277783186432], [-87.60632260352641, 41.82278356308904], [-87.60630233682008, 41.822789559885024], [-87.60628221277028, 41.82279582048222], [-87.60626223741507, 41.82280234311821], [-87.6062424168028, 41.822809125130334], [-87.60622275817514, 41.8228161647638], [-87.60620326757022, 41.822823460256195], [-87.60618394862924, 41.82283100892967], [-87.6061357829986, 41.82285126887031], [-87.60489865036251, 41.82326907790459], [-87.60488618404133, 41.823273092730936], [-87.60487521949304, 41.823276932508655], [-87.60486278852834, 41.823281650728966], [-87.60484930661205, 41.82328723021869], [-87.60483704714119, 41.823292747232735], [-87.6048271855152, 41.82329751145608], [-87.6048184078212, 41.8233020088474], [-87.60481037940755, 41.823306348027266], [-87.60480191461397, 41.82331116882633], [-87.60479333766806, 41.82331632654415], [-87.6047855007208, 41.823321295379984], [-87.6047572327323, 41.823341526083084], [-87.60471652058943, 41.82336869605984], [-87.60470052458207, 41.823382623822745], [-87.60468485482315, 41.82339675893244], [-87.60466951859557, 41.82341109603318], [-87.60465451835765, 41.823425630638965], [-87.6046398601683, 41.82344035918691], [-87.60462554648588, 41.82345527719107], [-87.60461158337955, 41.82347038018828], [-87.60459797573527, 41.82348566190726], [-87.60458472599103, 41.823501119662524], [-87.60457183902265, 41.82351674808307], [-87.60455931849212, 41.82353254269051], [-87.6045471692855, 41.82354849721349], [-87.60453539263716, 41.823564608958954], [-87.60452399584045, 41.823580871670806], [-87.60451297774297, 41.82359728084015], [-87.60450234562784, 41.82361383111117], [-87.60449210196373, 41.8236305170976], [-87.60448224799534, 41.823647335206], [-87.60447278860879, 41.823664279165065], [-87.60446372506924, 41.823681343580795], [-87.60445506224238, 41.82369852398245], [-87.6044468013934, 41.823715814976026], [-87.6044389437976, 41.82373321026731], [-87.60443149431059, 41.82375070628574], [-87.60442445419751, 41.823768297637386], [-87.6044178259476, 41.823785977135316], [-87.6044116108056, 41.823803741186076], [-87.60440581126073, 41.82382158260278], [-87.60440042855778, 41.823839497791994], [-87.60439546517577, 41.82385748046702], [-87.60439092117632, 41.823875525226285], [-87.60438680023185, 41.823893626690996], [-87.60438310121057, 41.82391177855161], [-87.60437982657116, 41.82392997632201], [-87.60437697757878, 41.82394821460817], [-87.60437455311194, 41.82396648620023], [-87.60437255682261, 41.82398478752], [-87.60437098758929, 41.824003111357584], [-87.60436926671751, 41.82403533381279], [-87.60435230548126, 41.82416287487605]]]</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DREXEL BLVD</t>
+          <t>COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DREXEL</t>
+          <t>COTTAGE GROVE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -17438,22 +17438,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>E HYDE PARK BLVD</t>
+          <t>E PERSHING RD</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>E OAKWOOD BLVD</t>
+          <t>E 35TH ST</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Buffered Bike Lane</t>
+          <t>Bike Lane</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>1.44027790321</t>
+          <t>0.535169697043</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -17473,19 +17473,19 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>[[[-87.6061357829986, 41.82285126887031], [-87.60609798571573, 41.82276399646166], [-87.60590091255791, 41.82238247366579], [-87.60556669332729, 41.8218485016191], [-87.60530502182334, 41.82143367779866], [-87.60503607482781, 41.82100731247258], [-87.6048651023532, 41.820736412610586], [-87.60468547053425, 41.82045272301633], [-87.60449083328942, 41.820146654278034], [-87.6044256482468, 41.820039488053965], [-87.60440298975179, 41.8199636312076], [-87.60436493891923, 41.819611683642336], [-87.60429991730739, 41.819055419679465], [-87.60429380433658, 41.81900362340333], [-87.60426189555417, 41.8187247681738], [-87.60423424833219, 41.81848098336986], [-87.60420878995686, 41.81825126419623], [-87.60417455131629, 41.817968413673675], [-87.60415552556421, 41.81781123864321], [-87.60413394449134, 41.81761153828346], [-87.60411028125793, 41.81739508449601], [-87.6040885112337, 41.8171992256062], [-87.6040700938691, 41.81703439693089], [-87.60405800489534, 41.81683774595473], [-87.60404268597567, 41.816588553468314], [-87.60403709666593, 41.81630849303128], [-87.60403120520014, 41.8160161354863], [-87.60402385839835, 41.81570661792346], [-87.6040170517352, 41.81545621443974], [-87.60400794890579, 41.81501570099713], [-87.60400263005133, 41.814758282399495], [-87.6039971166536, 41.8145069813334], [-87.60399159427311, 41.81425010973378], [-87.60398593909036, 41.81399836927459], [-87.60398044110272, 41.813765236437085], [-87.60397499985255, 41.81352699896516], [-87.60396816319397, 41.813199599950835], [-87.60396389986742, 41.8129954454885], [-87.60395896340789, 41.81276777679964], [-87.60395507075744, 41.812587068895915], [-87.60395103323813, 41.81239971908291], [-87.60394749744123, 41.81224261431615], [-87.60394634625938, 41.812192497109486], [-87.60394481883999, 41.812126322466376], [-87.60393970922209, 41.8119040592473], [-87.60393553325102, 41.81172255360749], [-87.60392887286369, 41.811376458031624], [-87.60392551762324, 41.81120206585357], [-87.6039220751111, 41.811026987049004], [-87.60391755623571, 41.81080453486339], [-87.60391271281719, 41.810565396211956], [-87.60390920747359, 41.810395859547214], [-87.60390545674095, 41.810224510714114], [-87.6039029260037, 41.810108878818895], [-87.60389805780825, 41.80989781291501], [-87.60389154426316, 41.80955704103505], [-87.60388737756344, 41.80933909368288], [-87.6038839679615, 41.80921055686321], [-87.60387961854272, 41.80904658706937], [-87.60387371153965, 41.80877837916568], [-87.60386741299754, 41.80847998089812], [-87.60386217213637, 41.80822741989517], [-87.60385829065206, 41.80802316594071], [-87.60385239269901, 41.80773868420216], [-87.60384783613233, 41.80751883906607], [-87.60384274399121, 41.807243419051346], [-87.60383646805631, 41.80693986273583], [-87.60383088501047, 41.80664640914328], [-87.6038268275711, 41.80644791716319], [-87.60381920996646, 41.8061785179137], [-87.60381478491121, 41.80591612025036], [-87.60381184231792, 41.80574166480126], [-87.60380626616268, 41.80551868439242], [-87.60380179621455, 41.80533089313059], [-87.60379613662855, 41.80512799991602], [-87.60379079943327, 41.80490019151557], [-87.6037865313686, 41.80469439808748], [-87.6037805331614, 41.80445368703591], [-87.60377677465617, 41.804267683853766], [-87.60377404877609, 41.80410075937107], [-87.60377006455334, 41.80385690535313], [-87.60376813499602, 41.80374251152941], [-87.60376478430065, 41.80361114875377], [-87.60375648729162, 41.803366141884204], [-87.60375141035728, 41.80319294589922], [-87.60374820447251, 41.803022835593254], [-87.60374626819105, 41.80289938597228], [-87.60374406398431, 41.80276709679405], [-87.603741005496, 41.802597042333126], [-87.60377786306702, 41.802278554577875]]]</t>
+          <t>[[[-87.61062764640718, 41.83117833227938], [-87.61056121164148, 41.8309831537708], [-87.61049735143008, 41.83088969918398], [-87.61035664310229, 41.830683783743886], [-87.61021807070779, 41.83042154772161], [-87.60976457816737, 41.82954607123712], [-87.60957313929535, 41.82921206775326], [-87.60953484063897, 41.829123898452686], [-87.60947872228488, 41.82899470323354], [-87.60920191148996, 41.828461613639654], [-87.60903435707688, 41.82813505890052], [-87.60893989467102, 41.82795095517259], [-87.60881964632634, 41.82771437489353], [-87.60875245248874, 41.82758217879819], [-87.60848246060718, 41.827057116463294], [-87.60835626491398, 41.82681471429994], [-87.6082719086208, 41.82665265487381], [-87.60807609502977, 41.82626881297509], [-87.60797191429859, 41.82606348435161], [-87.6079087205916, 41.82593893804116], [-87.60784009873232, 41.82580134557496], [-87.60760573951933, 41.82534195692333], [-87.60750781352307, 41.825147209548874], [-87.6073738248817, 41.824880744701375], [-87.60728073042753, 41.82469689396191], [-87.6071500174633, 41.824439506146774], [-87.60686734794898, 41.8239569091955]]]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MARTIN LUTHER KING JR DR</t>
+          <t>31ST DR</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MARTIN LUTHER KING JR</t>
+          <t>31ST</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -17495,22 +17495,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>E GARFIELD BLVD</t>
+          <t>S MOE DR</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>E 51ST ST</t>
+          <t>S FORT DEARBORN</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0.525487613949</t>
+          <t>0.112279352219</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -17530,19 +17530,19 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>[[[-87.61610503358958, 41.80209463506868], [-87.6161372553474, 41.80190169269912], [-87.61614074146709, 41.80158907436339], [-87.61612777562215, 41.80089368105505], [-87.61611061011892, 41.80022228554601], [-87.6161072447521, 41.80009063210527], [-87.61609367670414, 41.799567542526496], [-87.61608066594823, 41.799007655365806], [-87.61607252526402, 41.798655650381], [-87.61607043851457, 41.798547458174994], [-87.6160678890834, 41.798457127876596], [-87.61605837110685, 41.79805028367454], [-87.61604192712679, 41.79739045646684], [-87.6160235286314, 41.79670545121182], [-87.61602194699849, 41.79663990734271], [-87.61601550198797, 41.7963728214937], [-87.61599616418324, 41.79563948379497], [-87.61599287316523, 41.795514680599055], [-87.61597940877292, 41.795011981545464], [-87.6159753641248, 41.794792923748744], [-87.6159725954511, 41.7946429706259], [-87.61596722873355, 41.79447924837816]]]</t>
+          <t>[[[-87.60986250664294, 41.83853270823932], [-87.6095086258396, 41.83853049214663], [-87.60918890021458, 41.83853812491465], [-87.60875811449299, 41.83854840731297], [-87.60865431875239, 41.83855088477592], [-87.60833750976242, 41.838558445341555], [-87.60824493561356, 41.83856065473611], [-87.60779764356145, 41.83857132811791], [-87.60768798164275, 41.83857394411922]]]</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>31ST ST</t>
+          <t>OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>31ST</t>
+          <t>OAKWOOD</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -17552,22 +17552,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>E PERSHING RD</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>S MOE DR</t>
+          <t>LAKESHORE DR</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.374564177222</t>
+          <t>0.265190300727</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -17587,19 +17587,19 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>[[[-87.61711743673902, 41.83841544388878], [-87.61349382112748, 41.83846417399243], [-87.61336507987872, 41.8384654324603], [-87.61170778684063, 41.8384964974145], [-87.6113260948113, 41.838513422816135], [-87.61122239818451, 41.83851802083818], [-87.61106328407865, 41.83852507577069], [-87.61079286825503, 41.83852833767229], [-87.61023646107017, 41.83853504871899], [-87.61004517815752, 41.83853385151719], [-87.60986250664294, 41.83853270823932]]]</t>
+          <t>[[[-87.60435230548126, 41.82416287487605], [-87.60430631831143, 41.82416402356607], [-87.60428716161914, 41.824162095879494], [-87.60426796236939, 41.824160418216486], [-87.60424872656984, 41.824158991515496], [-87.6042294614419, 41.82415781582236], [-87.60421017058603, 41.824156892060216], [-87.60419086242726, 41.824156220282596], [-87.60417154057622, 41.82415580051237], [-87.60415221225436, 41.824155632795396], [-87.60413288226572, 41.82415571806249], [-87.60411355904553, 41.824156055466894], [-87.60409424500084, 41.824156645023855], [-87.60407494855669, 41.82415748678687], [-87.60405567333392, 41.82415857987863], [-87.60403642775758, 41.82415992435258], [-87.60401721664196, 41.82416152023936], [-87.60399804481145, 41.82416336666922], [-87.60397216606508, 41.82416626443172], [-87.60346372774372, 41.82428645007398], [-87.60283279718537, 41.82449961768677], [-87.60254227296632, 41.82459826474106], [-87.60246449645898, 41.82463065780316], [-87.60214041957721, 41.82476563187484], [-87.6020952755735, 41.8247849900892], [-87.6017964676506, 41.824913114836825], [-87.60160828555927, 41.824988222508935], [-87.60150680968545, 41.82502872373627], [-87.60091462496219, 41.825188150840695], [-87.60074975423764, 41.82519086558529], [-87.60046891563478, 41.82526537949098], [-87.60036960542857, 41.82529172834911], [-87.60027660609322, 41.82531640313449], [-87.59999145364394, 41.825392060591405], [-87.59984691458156, 41.8254304090753], [-87.5996240077739, 41.825489550046555], [-87.5995963400068, 41.82550927640572]]]</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>33RD ST</t>
+          <t>31ST ST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>33RD</t>
+          <t>31ST</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -17609,22 +17609,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>S STATE ST</t>
+          <t>S MICHIGAN AVE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>S GILES AVE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Marked Shared Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0.47034639757</t>
+          <t>0.204433765585</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -17644,19 +17644,19 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>[[[-87.62649453439884, 41.834657620039394], [-87.6261375484813, 41.834653255468275], [-87.62598820768505, 41.834655523097894], [-87.6258713558933, 41.83465729648271], [-87.62555479911322, 41.834663112644094], [-87.62521987635559, 41.834667222892755], [-87.62505539738287, 41.834670172980104], [-87.62490108129768, 41.834672941521305], [-87.62458217233613, 41.834675666707916], [-87.62423396810284, 41.83467955437231], [-87.62419467526055, 41.83468228203092], [-87.62332410153712, 41.834694699177206], [-87.6225766889668, 41.834705354550316], [-87.62204427228347, 41.83471294207457], [-87.62183407802331, 41.834710293288616], [-87.62162465056676, 41.834707653371126], [-87.62122627094816, 41.83471231672194], [-87.62080305524594, 41.834717269393636], [-87.62061503357474, 41.834712419521736], [-87.62049200866362, 41.83470924673693], [-87.6196388712932, 41.834730650392935], [-87.61940523053126, 41.834732824088015], [-87.61923746068237, 41.8347343849626], [-87.61879845501683, 41.83473992804518], [-87.61849043146212, 41.83474381686139], [-87.61818788325031, 41.83474705287812], [-87.61738398483341, 41.83475564899769]]]</t>
+          <t>[[[-87.62343694336933, 41.83833704540958], [-87.62323358361407, 41.83833847406264], [-87.6219191008301, 41.838356765893344], [-87.62177979242179, 41.83835870302541], [-87.62128211303167, 41.83836481491048], [-87.62100750971918, 41.8383681865488], [-87.62063024755903, 41.83837298145963], [-87.62047048387781, 41.83837500885838], [-87.62015738391769, 41.83837922174425], [-87.61999021695806, 41.83838147080919], [-87.61947655373596, 41.838387441384285]]]</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>OAKWOOD BLVD</t>
+          <t>35TH ST</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>OAKWOOD</t>
+          <t>35TH</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -17666,12 +17666,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>S COTTAGE GROVE AVE</t>
+          <t>S INDIANA AVE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>E PERSHING RD</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -17681,7 +17681,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.179532699715</t>
+          <t>0.247640012693</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -17701,19 +17701,19 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>[[[-87.60684961994563, 41.822720681391324], [-87.60679180817826, 41.82272115395717], [-87.60677001340125, 41.82272103500519], [-87.60674821900858, 41.82272120146208], [-87.60672643224186, 41.822721651572905], [-87.60670465910856, 41.822722386276055], [-87.60668290562634, 41.822723405609615], [-87.60666118024034, 41.82272470782627], [-87.60663948895807, 41.82272629386447], [-87.60661783660379, 41.82272816285434], [-87.60659623160228, 41.822730314849224], [-87.60657467999161, 41.822732748086665], [-87.60655318900317, 41.82273546171211], [-87.60653176465463, 41.82273845576364], [-87.60651041297386, 41.822741729379096], [-87.6064891412025, 41.82274528080366], [-87.60646795535817, 41.82274911007541], [-87.60644686148913, 41.82275321453169], [-87.60642586802022, 41.8227575942258], [-87.60640497858236, 41.82276224738011], [-87.60638420162077, 41.82276717224742], [-87.6063635431735, 41.82277236706532], [-87.60634300805471, 41.82277783186432], [-87.60632260352641, 41.82278356308904], [-87.60630233682008, 41.822789559885024], [-87.60628221277028, 41.82279582048222], [-87.60626223741507, 41.82280234311821], [-87.6062424168028, 41.822809125130334], [-87.60622275817514, 41.8228161647638], [-87.60620326757022, 41.822823460256195], [-87.60618394862924, 41.82283100892967], [-87.6061357829986, 41.82285126887031], [-87.60489865036251, 41.82326907790459], [-87.60488618404133, 41.823273092730936], [-87.60487521949304, 41.823276932508655], [-87.60486278852834, 41.823281650728966], [-87.60484930661205, 41.82328723021869], [-87.60483704714119, 41.823292747232735], [-87.6048271855152, 41.82329751145608], [-87.6048184078212, 41.8233020088474], [-87.60481037940755, 41.823306348027266], [-87.60480191461397, 41.82331116882633], [-87.60479333766806, 41.82331632654415], [-87.6047855007208, 41.823321295379984], [-87.6047572327323, 41.823341526083084], [-87.60471652058943, 41.82336869605984], [-87.60470052458207, 41.823382623822745], [-87.60468485482315, 41.82339675893244], [-87.60466951859557, 41.82341109603318], [-87.60465451835765, 41.823425630638965], [-87.6046398601683, 41.82344035918691], [-87.60462554648588, 41.82345527719107], [-87.60461158337955, 41.82347038018828], [-87.60459797573527, 41.82348566190726], [-87.60458472599103, 41.823501119662524], [-87.60457183902265, 41.82351674808307], [-87.60455931849212, 41.82353254269051], [-87.6045471692855, 41.82354849721349], [-87.60453539263716, 41.823564608958954], [-87.60452399584045, 41.823580871670806], [-87.60451297774297, 41.82359728084015], [-87.60450234562784, 41.82361383111117], [-87.60449210196373, 41.8236305170976], [-87.60448224799534, 41.823647335206], [-87.60447278860879, 41.823664279165065], [-87.60446372506924, 41.823681343580795], [-87.60445506224238, 41.82369852398245], [-87.6044468013934, 41.823715814976026], [-87.6044389437976, 41.82373321026731], [-87.60443149431059, 41.82375070628574], [-87.60442445419751, 41.823768297637386], [-87.6044178259476, 41.823785977135316], [-87.6044116108056, 41.823803741186076], [-87.60440581126073, 41.82382158260278], [-87.60440042855778, 41.823839497791994], [-87.60439546517577, 41.82385748046702], [-87.60439092117632, 41.823875525226285], [-87.60438680023185, 41.823893626690996], [-87.60438310121057, 41.82391177855161], [-87.60437982657116, 41.82392997632201], [-87.60437697757878, 41.82394821460817], [-87.60437455311194, 41.82396648620023], [-87.60437255682261, 41.82398478752], [-87.60437098758929, 41.824003111357584], [-87.60436926671751, 41.82403533381279], [-87.60435230548126, 41.82416287487605]]]</t>
+          <t>[[[-87.62175790723948, 41.83105114677236], [-87.62147204346718, 41.83105439399251], [-87.62114680081156, 41.83105756560645], [-87.62071506301695, 41.83106177458682], [-87.62054500801808, 41.83106270827247], [-87.62038410991939, 41.83106359050268], [-87.61993842551381, 41.831068138560155], [-87.61959497831648, 41.83107164288365], [-87.61932790430228, 41.83107429835225], [-87.6192145415096, 41.83107542490796], [-87.61861331357758, 41.831080192721124], [-87.61840049624368, 41.8310834879503], [-87.61811354507196, 41.8310879292089], [-87.61794575632707, 41.83109052619566], [-87.61760482133919, 41.83109575717714], [-87.61730766754923, 41.83109415363711], [-87.61696083107093, 41.83109228088914]]]</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>COTTAGE GROVE AVE</t>
+          <t>35TH ST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>COTTAGE GROVE</t>
+          <t>35TH</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -17723,22 +17723,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>E PERSHING RD</t>
+          <t>S STATE ST</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>E 35TH ST</t>
+          <t>S INDIANA AVE</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Marked Shared Lane</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0.535169697043</t>
+          <t>0.251982034456</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -17758,19 +17758,19 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>[[[-87.61062764640718, 41.83117833227938], [-87.61056121164148, 41.8309831537708], [-87.61049735143008, 41.83088969918398], [-87.61035664310229, 41.830683783743886], [-87.61021807070779, 41.83042154772161], [-87.60976457816737, 41.82954607123712], [-87.60957313929535, 41.82921206775326], [-87.60953484063897, 41.829123898452686], [-87.60947872228488, 41.82899470323354], [-87.60920191148996, 41.828461613639654], [-87.60903435707688, 41.82813505890052], [-87.60893989467102, 41.82795095517259], [-87.60881964632634, 41.82771437489353], [-87.60875245248874, 41.82758217879819], [-87.60848246060718, 41.827057116463294], [-87.60835626491398, 41.82681471429994], [-87.6082719086208, 41.82665265487381], [-87.60807609502977, 41.82626881297509], [-87.60797191429859, 41.82606348435161], [-87.6079087205916, 41.82593893804116], [-87.60784009873232, 41.82580134557496], [-87.60760573951933, 41.82534195692333], [-87.60750781352307, 41.825147209548874], [-87.6073738248817, 41.824880744701375], [-87.60728073042753, 41.82469689396191], [-87.6071500174633, 41.824439506146774], [-87.60686734794898, 41.8239569091955]]]</t>
+          <t>[[[-87.6266385987239, 41.83100580881331], [-87.6264732958851, 41.83101107967687], [-87.62623318245583, 41.83101873668085], [-87.62601026219642, 41.831016431371204], [-87.62591536563151, 41.83101335928809], [-87.62580089456586, 41.83100965335254], [-87.62578894519758, 41.8310097769209], [-87.62528748091881, 41.83101497359384], [-87.62497040535462, 41.83101825860181], [-87.62460523369673, 41.83102204008217], [-87.62425145860854, 41.831023753331884], [-87.62423505388152, 41.83102409322796], [-87.62325146933688, 41.831035886002816], [-87.623068985482, 41.831038072800894], [-87.62257009356864, 41.831042925980455], [-87.62249985576759, 41.831043609555515], [-87.62195505561091, 41.831048907025604], [-87.62175790723948, 41.83105114677236]]]</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>31ST DR</t>
+          <t>PERSHING RD</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>31ST</t>
+          <t>PERSHING</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -17780,22 +17780,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>S MOE DR</t>
+          <t>S MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>S FORT DEARBORN</t>
+          <t>S COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Buffered Bike Lane</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0.112279352219</t>
+          <t>0.52273584865</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -17815,19 +17815,19 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>[[[-87.60986250664294, 41.83853270823932], [-87.6095086258396, 41.83853049214663], [-87.60918890021458, 41.83853812491465], [-87.60875811449299, 41.83854840731297], [-87.60865431875239, 41.83855088477592], [-87.60833750976242, 41.838558445341555], [-87.60824493561356, 41.83856065473611], [-87.60779764356145, 41.83857132811791], [-87.60768798164275, 41.83857394411922]]]</t>
+          <t>[[[-87.61699111101917, 41.82382621643897], [-87.61672658426848, 41.823830247623874], [-87.61611742079225, 41.823839530348515], [-87.61610351380473, 41.8238397010112], [-87.6154691158385, 41.82384748030514], [-87.61514202830347, 41.82385149048068], [-87.61435832379438, 41.82386109676443], [-87.61307015328607, 41.82387688472249], [-87.61261856025574, 41.82388291330555], [-87.61213034165046, 41.82388942863265], [-87.61127647198559, 41.82389814834697], [-87.61055372981066, 41.82390552337138], [-87.60983565600785, 41.82391284582243], [-87.60958135685671, 41.82391543849396], [-87.6083907741053, 41.82392832878097], [-87.60833202655425, 41.82392896457945], [-87.60732163043673, 41.82394102449633], [-87.60702288161544, 41.823950057947265], [-87.60691033374472, 41.82395217241693], [-87.60686734794898, 41.8239569091955]]]</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>OAKWOOD BLVD</t>
+          <t>PERSHING RD</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>OAKWOOD</t>
+          <t>PERSHING</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -17837,12 +17837,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>E PERSHING RD</t>
+          <t>S COTTAGE GROVE AVE</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>LAKESHORE DR</t>
+          <t>E OAKWOOD BLVD</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -17852,7 +17852,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0.265190300727</t>
+          <t>0.135533728291</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -17872,7 +17872,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>[[[-87.60435230548126, 41.82416287487605], [-87.60430631831143, 41.82416402356607], [-87.60428716161914, 41.824162095879494], [-87.60426796236939, 41.824160418216486], [-87.60424872656984, 41.824158991515496], [-87.6042294614419, 41.82415781582236], [-87.60421017058603, 41.824156892060216], [-87.60419086242726, 41.824156220282596], [-87.60417154057622, 41.82415580051237], [-87.60415221225436, 41.824155632795396], [-87.60413288226572, 41.82415571806249], [-87.60411355904553, 41.824156055466894], [-87.60409424500084, 41.824156645023855], [-87.60407494855669, 41.82415748678687], [-87.60405567333392, 41.82415857987863], [-87.60403642775758, 41.82415992435258], [-87.60401721664196, 41.82416152023936], [-87.60399804481145, 41.82416336666922], [-87.60397216606508, 41.82416626443172], [-87.60346372774372, 41.82428645007398], [-87.60283279718537, 41.82449961768677], [-87.60254227296632, 41.82459826474106], [-87.60246449645898, 41.82463065780316], [-87.60214041957721, 41.82476563187484], [-87.6020952755735, 41.8247849900892], [-87.6017964676506, 41.824913114836825], [-87.60160828555927, 41.824988222508935], [-87.60150680968545, 41.82502872373627], [-87.60091462496219, 41.825188150840695], [-87.60074975423764, 41.82519086558529], [-87.60046891563478, 41.82526537949098], [-87.60036960542857, 41.82529172834911], [-87.60027660609322, 41.82531640313449], [-87.59999145364394, 41.825392060591405], [-87.59984691458156, 41.8254304090753], [-87.5996240077739, 41.825489550046555], [-87.5995963400068, 41.82550927640572]]]</t>
+          <t>[[[-87.60686734794898, 41.8239569091955], [-87.60606651814183, 41.82417374136248], [-87.60576295911753, 41.82426465478336], [-87.60574292254485, 41.82427037292759], [-87.60572275653709, 41.824275828247], [-87.60570246591914, 41.82428101987172], [-87.60568205673985, 41.82428594513898], [-87.60566153743501, 41.824290603201796], [-87.60564091042225, 41.82429499317505], [-87.60562018535114, 41.824299113319164], [-87.60559936705677, 41.82430296186401], [-87.6055784615575, 41.824306538847644], [-87.60555747730946, 41.8243098416226], [-87.60553641792379, 41.8243128702117], [-87.60551529184642, 41.824315622867694], [-87.6054675496305, 41.82432080616751], [-87.60514959326278, 41.82431298815248], [-87.60506702606838, 41.82430186758017], [-87.60498473109828, 41.8242896709576], [-87.60490273359159, 41.824276402046785], [-87.60482105759388, 41.82426206370194], [-87.60473921548223, 41.8242465609951], [-87.6045999908213, 41.824210864913994], [-87.60435230548126, 41.82416287487605]]]</t>
         </is>
       </c>
     </row>
@@ -17894,12 +17894,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>S MICHIGAN AVE</t>
+          <t>S GILES AVE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>S GILES AVE</t>
+          <t>S DR MARTIN LUTHER KING JR DR</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -17909,7 +17909,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0.204433765585</t>
+          <t>0.121774289186</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -17929,19 +17929,19 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>[[[-87.62343694336933, 41.83833704540958], [-87.62323358361407, 41.83833847406264], [-87.6219191008301, 41.838356765893344], [-87.62177979242179, 41.83835870302541], [-87.62128211303167, 41.83836481491048], [-87.62100750971918, 41.8383681865488], [-87.62063024755903, 41.83837298145963], [-87.62047048387781, 41.83837500885838], [-87.62015738391769, 41.83837922174425], [-87.61999021695806, 41.83838147080919], [-87.61947655373596, 41.838387441384285]]]</t>
+          <t>[[[-87.61947655373596, 41.838387441384285], [-87.61826297733084, 41.83840128373133], [-87.61746126495309, 41.838411426314124], [-87.61711743673902, 41.83841544388878]]]</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>35TH ST</t>
+          <t>PAYNE DR</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>35TH</t>
+          <t>PAYNE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -17951,22 +17951,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>S INDIANA AVE</t>
+          <t>E RAINEY DR</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>E 55TH ST</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Bike Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0.247640012693</t>
+          <t>0.0675160768248</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -17986,54 +17986,54 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>[[[-87.62175790723948, 41.83105114677236], [-87.62147204346718, 41.83105439399251], [-87.62114680081156, 41.83105756560645], [-87.62071506301695, 41.83106177458682], [-87.62054500801808, 41.83106270827247], [-87.62038410991939, 41.83106359050268], [-87.61993842551381, 41.831068138560155], [-87.61959497831648, 41.83107164288365], [-87.61932790430228, 41.83107429835225], [-87.6192145415096, 41.83107542490796], [-87.61861331357758, 41.831080192721124], [-87.61840049624368, 41.8310834879503], [-87.61811354507196, 41.8310879292089], [-87.61794575632707, 41.83109052619566], [-87.61760482133919, 41.83109575717714], [-87.61730766754923, 41.83109415363711], [-87.61696083107093, 41.83109228088914]]]</t>
+          <t>[[[-87.60737728719235, 41.79496310174033], [-87.60739572258301, 41.79490141710621], [-87.60759032740498, 41.794597181214684], [-87.60781895881487, 41.79429315897816], [-87.60788597312641, 41.79420071616683], [-87.60793532745689, 41.79414594962413], [-87.60799024123432, 41.794105496864226]]]</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>35TH ST</t>
+          <t>55TH PL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>35TH</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>S STATE ST</t>
+          <t>E 55TH ST</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>S INDIANA AVE</t>
+          <t>S DORCHESTER AVE</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Marked Shared Lane</t>
+          <t>Protected Bike Lane</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0.251982034456</t>
+          <t>0.0456951713071</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2W</t>
+          <t>1W</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -18043,34 +18043,34 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>[[[-87.6266385987239, 41.83100580881331], [-87.6264732958851, 41.83101107967687], [-87.62623318245583, 41.83101873668085], [-87.62601026219642, 41.831016431371204], [-87.62591536563151, 41.83101335928809], [-87.62580089456586, 41.83100965335254], [-87.62578894519758, 41.8310097769209], [-87.62528748091881, 41.83101497359384], [-87.62497040535462, 41.83101825860181], [-87.62460523369673, 41.83102204008217], [-87.62425145860854, 41.831023753331884], [-87.62423505388152, 41.83102409322796], [-87.62325146933688, 41.831035886002816], [-87.623068985482, 41.831038072800894], [-87.62257009356864, 41.831042925980455], [-87.62249985576759, 41.831043609555515], [-87.62195505561091, 41.831048907025604], [-87.62175790723948, 41.83105114677236]]]</t>
+          <t>[[[-87.59230182841584, 41.795115630665705], [-87.59228479651814, 41.79504607209104], [-87.59225548130618, 41.79497654411554], [-87.59219846154255, 41.79489528677071], [-87.59216267495331, 41.79487450803364], [-87.5920133591238, 41.794803290937494], [-87.59193680903836, 41.794782379617466], [-87.59185276036327, 41.794775717447465], [-87.59167067344248, 41.79477653357941]]]</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PERSHING RD</t>
+          <t>55TH PL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PERSHING</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>S MARTIN LUTHER KING JR DR</t>
+          <t>S DORCHESTER AVE</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>S COTTAGE GROVE AVE</t>
+          <t>E 55TH ST</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -18080,17 +18080,17 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.52273584865</t>
+          <t>0.144696496175</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2W</t>
+          <t>1W</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -18100,19 +18100,19 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>[[[-87.61699111101917, 41.82382621643897], [-87.61672658426848, 41.823830247623874], [-87.61611742079225, 41.823839530348515], [-87.61610351380473, 41.8238397010112], [-87.6154691158385, 41.82384748030514], [-87.61514202830347, 41.82385149048068], [-87.61435832379438, 41.82386109676443], [-87.61307015328607, 41.82387688472249], [-87.61261856025574, 41.82388291330555], [-87.61213034165046, 41.82388942863265], [-87.61127647198559, 41.82389814834697], [-87.61055372981066, 41.82390552337138], [-87.60983565600785, 41.82391284582243], [-87.60958135685671, 41.82391543849396], [-87.6083907741053, 41.82392832878097], [-87.60833202655425, 41.82392896457945], [-87.60732163043673, 41.82394102449633], [-87.60702288161544, 41.823950057947265], [-87.60691033374472, 41.82395217241693], [-87.60686734794898, 41.8239569091955]]]</t>
+          <t>[[[-87.59167067344248, 41.79477653357941], [-87.59136866354801, 41.79477788763556], [-87.59102905319932, 41.7947802494273], [-87.5907804071988, 41.794781030192134], [-87.59057041516495, 41.79478167500291], [-87.59032230194119, 41.79478403653916], [-87.59011020296843, 41.79478605342406], [-87.58985624501801, 41.79478954209586], [-87.58964247007485, 41.794793948510694], [-87.58954419795131, 41.79480903782709], [-87.5894761210009, 41.79482602245259], [-87.5894100443973, 41.7948539709812], [-87.58930529537159, 41.794916096688844], [-87.58922782297005, 41.79504082853871], [-87.58920177375734, 41.79511475522187], [-87.58919925975736, 41.795164108872186], [-87.58920472557244, 41.79519313923364]]]</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PERSHING RD</t>
+          <t>55TH ST</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PERSHING</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -18122,12 +18122,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>S COTTAGE GROVE AVE</t>
+          <t>E 55TH PL</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>E OAKWOOD BLVD</t>
+          <t>S LAKE PARK AVE</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -18137,7 +18137,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0.135533728291</t>
+          <t>0.0858058887654</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -18157,19 +18157,19 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>[[[-87.60686734794898, 41.8239569091955], [-87.60606651814183, 41.82417374136248], [-87.60576295911753, 41.82426465478336], [-87.60574292254485, 41.82427037292759], [-87.60572275653709, 41.824275828247], [-87.60570246591914, 41.82428101987172], [-87.60568205673985, 41.82428594513898], [-87.60566153743501, 41.824290603201796], [-87.60564091042225, 41.82429499317505], [-87.60562018535114, 41.824299113319164], [-87.60559936705677, 41.82430296186401], [-87.6055784615575, 41.824306538847644], [-87.60555747730946, 41.8243098416226], [-87.60553641792379, 41.8243128702117], [-87.60551529184642, 41.824315622867694], [-87.6054675496305, 41.82432080616751], [-87.60514959326278, 41.82431298815248], [-87.60506702606838, 41.82430186758017], [-87.60498473109828, 41.8242896709576], [-87.60490273359159, 41.824276402046785], [-87.60482105759388, 41.82426206370194], [-87.60473921548223, 41.8242465609951], [-87.6045999908213, 41.824210864913994], [-87.60435230548126, 41.82416287487605]]]</t>
+          <t>[[[-87.58920472557244, 41.79519313923364], [-87.58843978013414, 41.795185708334266], [-87.58754346134559, 41.795176995453275]]]</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>31ST ST</t>
+          <t>55TH ST</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>31ST</t>
+          <t>55TH</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -18179,22 +18179,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>S GILES AVE</t>
+          <t>S LAKE PARK AVE</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>S DR MARTIN LUTHER KING JR DR</t>
+          <t>S HYDE PARK BLVD</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Protected Bike Lane</t>
+          <t>Marked Shared Lane</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0.121774289186</t>
+          <t>0.185855928634</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -18214,7 +18214,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>[[[-87.61947655373596, 41.838387441384285], [-87.61826297733084, 41.83840128373133], [-87.61746126495309, 41.838411426314124], [-87.61711743673902, 41.83841544388878]]]</t>
+          <t>[[[-87.58754346134559, 41.795176995453275], [-87.58738962534618, 41.795178680573635], [-87.58723653779546, 41.79518035774402], [-87.58718928018563, 41.79518087552708], [-87.587017867405, 41.79518275390326], [-87.58694172794344, 41.7951835872402], [-87.58690389104218, 41.795184002251354], [-87.58673557437942, 41.79518584540241], [-87.58671603381707, 41.795186059636485], [-87.58661850963912, 41.79518760010154], [-87.58616460134657, 41.79519476866744], [-87.58576988324349, 41.79519906136454], [-87.58540490313923, 41.795203699386356], [-87.58511445279412, 41.795207390147176], [-87.58484326462393, 41.795207078465104], [-87.58467848640464, 41.79520974297046], [-87.58451912941597, 41.795212320129835], [-87.58431745967604, 41.79521624722297], [-87.58394543361024, 41.795220065764205]]]</t>
         </is>
       </c>
     </row>

</xml_diff>